<commit_message>
feat: add HT/TTC toggle, fix D48 objective & optimize WhatsApp autofill
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2642,17 +2642,17 @@
         </is>
       </c>
       <c r="C2" s="85" t="n">
-        <v>11833</v>
+        <v>11834</v>
       </c>
       <c r="D2" s="85" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="195" t="n"/>
       <c r="F2" s="85" t="n">
-        <v>80610</v>
+        <v>80611</v>
       </c>
       <c r="G2" s="85" t="n">
-        <v>51885</v>
+        <v>51886</v>
       </c>
       <c r="H2" s="195" t="n">
         <v>0.55</v>
@@ -2664,7 +2664,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>-591</v>
+        <v>-1972</v>
       </c>
     </row>
     <row r="3">
@@ -2679,17 +2679,17 @@
         </is>
       </c>
       <c r="C3" s="83" t="n">
-        <v>30407</v>
+        <v>30408</v>
       </c>
       <c r="D3" s="83" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="82" t="n"/>
       <c r="F3" s="83" t="n">
-        <v>70174</v>
+        <v>70175</v>
       </c>
       <c r="G3" s="83" t="n">
-        <v>116700</v>
+        <v>116701</v>
       </c>
       <c r="H3" s="82" t="n">
         <v>-0.4</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>-1520</v>
+        <v>-5068</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="250">
@@ -2753,14 +2753,14 @@
         </is>
       </c>
       <c r="C5" s="83" t="n">
-        <v>4166</v>
+        <v>4167</v>
       </c>
       <c r="D5" s="83" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="82" t="n"/>
       <c r="F5" s="83" t="n">
-        <v>441682</v>
+        <v>441683</v>
       </c>
       <c r="G5" s="83" t="n">
         <v>66016</v>
@@ -2775,7 +2775,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>-208</v>
+        <v>-694</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="250">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="E6" s="82" t="n"/>
       <c r="F6" s="83" t="n">
-        <v>128161</v>
+        <v>128162</v>
       </c>
       <c r="G6" s="83" t="n">
         <v>251467</v>
@@ -2812,7 +2812,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>-342</v>
+        <v>-1141</v>
       </c>
     </row>
     <row r="7">
@@ -2837,7 +2837,7 @@
         <v>11491</v>
       </c>
       <c r="G7" s="83" t="n">
-        <v>11142</v>
+        <v>11143</v>
       </c>
       <c r="H7" s="82" t="n">
         <v>0.03</v>
@@ -2910,10 +2910,10 @@
       </c>
       <c r="E9" s="201" t="n"/>
       <c r="F9" s="80" t="n">
-        <v>2595019</v>
+        <v>2595020</v>
       </c>
       <c r="G9" s="80" t="n">
-        <v>2446914</v>
+        <v>2446915</v>
       </c>
       <c r="H9" s="201" t="n">
         <v>0.06</v>
@@ -2925,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>-8035</v>
+        <v>-26785</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="250">
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="C10" s="85" t="n">
-        <v>9515</v>
+        <v>9516</v>
       </c>
       <c r="D10" s="85" t="n">
         <v>9375</v>
@@ -2949,22 +2949,22 @@
         <v>0.01502015325954886</v>
       </c>
       <c r="F10" s="85" t="n">
-        <v>306923</v>
+        <v>306924</v>
       </c>
       <c r="G10" s="85" t="n">
-        <v>271247</v>
+        <v>271248</v>
       </c>
       <c r="H10" s="195" t="n">
         <v>0.13</v>
       </c>
       <c r="I10" s="85" t="n">
-        <v>4830</v>
+        <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>45000</v>
+        <v>11842</v>
       </c>
       <c r="K10" t="n">
-        <v>1774</v>
+        <v>388</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -2988,10 +2988,10 @@
         <v>-0.5039013379414876</v>
       </c>
       <c r="F11" s="83" t="n">
-        <v>44073</v>
+        <v>44074</v>
       </c>
       <c r="G11" s="83" t="n">
-        <v>47811</v>
+        <v>47812</v>
       </c>
       <c r="H11" s="82" t="n">
         <v>-0.08</v>
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K11" t="n">
-        <v>537</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="C12" s="83" t="n">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="D12" s="83" t="n">
         <v>5000</v>
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>24000</v>
+        <v>6316</v>
       </c>
       <c r="K12" t="n">
-        <v>1139</v>
+        <v>851</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="E13" s="82" t="n"/>
       <c r="F13" s="83" t="n">
-        <v>5617</v>
+        <v>5618</v>
       </c>
       <c r="G13" s="83" t="n">
         <v>1413</v>
@@ -3101,10 +3101,10 @@
       </c>
       <c r="E14" s="82" t="n"/>
       <c r="F14" s="83" t="n">
-        <v>2421</v>
+        <v>2422</v>
       </c>
       <c r="G14" s="83" t="n">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="H14" s="82" t="n">
         <v>2.04</v>
@@ -3218,22 +3218,22 @@
         <v>-0.2054502184307671</v>
       </c>
       <c r="F17" s="80" t="n">
-        <v>842195</v>
+        <v>842196</v>
       </c>
       <c r="G17" s="80" t="n">
-        <v>792555</v>
+        <v>792556</v>
       </c>
       <c r="H17" s="201" t="n">
         <v>0.06</v>
       </c>
       <c r="I17" s="80" t="n">
-        <v>10254</v>
+        <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>129999</v>
+        <v>34211</v>
       </c>
       <c r="K17" t="n">
-        <v>5424</v>
+        <v>2115</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3255,10 +3255,10 @@
       </c>
       <c r="E18" s="195" t="n"/>
       <c r="F18" s="85" t="n">
-        <v>2464</v>
+        <v>2465</v>
       </c>
       <c r="G18" s="85" t="n">
-        <v>5289</v>
+        <v>5290</v>
       </c>
       <c r="H18" s="195" t="n">
         <v>-0.53</v>
@@ -3332,7 +3332,7 @@
         <v>71</v>
       </c>
       <c r="G20" s="83" t="n">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="H20" s="82" t="n">
         <v>-0.96</v>
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="C21" s="83" t="n">
-        <v>9415</v>
+        <v>9416</v>
       </c>
       <c r="D21" s="83" t="n">
         <v>9375</v>
@@ -3371,19 +3371,19 @@
         <v>284205</v>
       </c>
       <c r="G21" s="83" t="n">
-        <v>243983</v>
+        <v>243984</v>
       </c>
       <c r="H21" s="82" t="n">
         <v>0.16</v>
       </c>
       <c r="I21" s="83" t="n">
-        <v>4640</v>
+        <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>45000</v>
+        <v>11842</v>
       </c>
       <c r="K21" t="n">
-        <v>1779</v>
+        <v>404</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3398,10 +3398,10 @@
         </is>
       </c>
       <c r="C22" s="83" t="n">
-        <v>6736</v>
+        <v>6737</v>
       </c>
       <c r="D22" s="83" t="n">
-        <v>7291</v>
+        <v>7292</v>
       </c>
       <c r="E22" s="82" t="n">
         <v>-0.07612617117745635</v>
@@ -3410,7 +3410,7 @@
         <v>138414</v>
       </c>
       <c r="G22" s="83" t="n">
-        <v>161010</v>
+        <v>161011</v>
       </c>
       <c r="H22" s="82" t="n">
         <v>-0.14</v>
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>35000</v>
+        <v>9211</v>
       </c>
       <c r="K22" t="n">
-        <v>1413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3449,19 +3449,19 @@
         <v>74113</v>
       </c>
       <c r="G23" s="83" t="n">
-        <v>55932</v>
+        <v>55933</v>
       </c>
       <c r="H23" s="82" t="n">
         <v>0.33</v>
       </c>
       <c r="I23" s="83" t="n">
-        <v>1755</v>
+        <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K23" t="n">
-        <v>447</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3518,13 +3518,13 @@
         <v>26882</v>
       </c>
       <c r="D25" s="80" t="n">
-        <v>26041</v>
+        <v>26042</v>
       </c>
       <c r="E25" s="201" t="n">
         <v>0.03228557088000006</v>
       </c>
       <c r="F25" s="80" t="n">
-        <v>748674</v>
+        <v>748675</v>
       </c>
       <c r="G25" s="80" t="n">
         <v>701828</v>
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>125000</v>
+        <v>32895</v>
       </c>
       <c r="K25" t="n">
-        <v>4905</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3554,10 +3554,10 @@
         </is>
       </c>
       <c r="C26" s="85" t="n">
-        <v>10329</v>
+        <v>10330</v>
       </c>
       <c r="D26" s="85" t="n">
-        <v>10416</v>
+        <v>10417</v>
       </c>
       <c r="E26" s="195" t="n">
         <v>-0.008346852500003554</v>
@@ -3566,19 +3566,19 @@
         <v>309112</v>
       </c>
       <c r="G26" s="85" t="n">
-        <v>357613</v>
+        <v>357614</v>
       </c>
       <c r="H26" s="195" t="n">
         <v>-0.14</v>
       </c>
       <c r="I26" s="85" t="n">
-        <v>3177</v>
+        <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>50000</v>
+        <v>13158</v>
       </c>
       <c r="K26" t="n">
-        <v>1983</v>
+        <v>471</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3593,7 +3593,7 @@
         </is>
       </c>
       <c r="C27" s="83" t="n">
-        <v>2883</v>
+        <v>2884</v>
       </c>
       <c r="D27" s="83" t="n">
         <v>2083</v>
@@ -3602,22 +3602,22 @@
         <v>0.3842271905517594</v>
       </c>
       <c r="F27" s="83" t="n">
-        <v>65298</v>
+        <v>65299</v>
       </c>
       <c r="G27" s="83" t="n">
-        <v>66045</v>
+        <v>66046</v>
       </c>
       <c r="H27" s="82" t="n">
         <v>-0.01</v>
       </c>
       <c r="I27" s="83" t="n">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K27" t="n">
-        <v>355</v>
+        <v>-42</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3641,7 +3641,7 @@
         <v>-0.20101332391284</v>
       </c>
       <c r="F28" s="83" t="n">
-        <v>230158</v>
+        <v>230159</v>
       </c>
       <c r="G28" s="83" t="n">
         <v>152407</v>
@@ -3650,13 +3650,13 @@
         <v>0.51</v>
       </c>
       <c r="I28" s="83" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K28" t="n">
-        <v>500</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3695,7 +3695,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>-628</v>
+        <v>-2096</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1" s="250">
@@ -3734,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>-318</v>
+        <v>-1062</v>
       </c>
     </row>
     <row r="31" ht="14.25" customHeight="1" s="250">
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c r="C31" s="83" t="n">
-        <v>4570</v>
+        <v>4571</v>
       </c>
       <c r="D31" s="83" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
         <v>53950</v>
       </c>
       <c r="G31" s="83" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H31" s="82" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>-228</v>
+        <v>-762</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="250">
@@ -3827,10 +3827,10 @@
         </is>
       </c>
       <c r="C33" s="80" t="n">
-        <v>54331</v>
+        <v>54332</v>
       </c>
       <c r="D33" s="80" t="n">
-        <v>29166</v>
+        <v>29167</v>
       </c>
       <c r="E33" s="201" t="n">
         <v>0.8628063901142835</v>
@@ -3845,13 +3845,13 @@
         <v>0.78</v>
       </c>
       <c r="I33" s="80" t="n">
-        <v>14695</v>
+        <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>140000</v>
+        <v>36842</v>
       </c>
       <c r="K33" t="n">
-        <v>4283</v>
+        <v>-2915</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3913,7 +3913,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="83" t="n">
-        <v>10617</v>
+        <v>10618</v>
       </c>
       <c r="H35" s="82" t="n">
         <v>-1</v>
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="83" t="n">
-        <v>7452</v>
+        <v>7453</v>
       </c>
       <c r="H36" s="82" t="n">
         <v>-1</v>
@@ -3989,7 +3989,7 @@
         <v>112871</v>
       </c>
       <c r="G37" s="83" t="n">
-        <v>381290</v>
+        <v>381291</v>
       </c>
       <c r="H37" s="82" t="n">
         <v>-0.7</v>
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>54999</v>
+        <v>14474</v>
       </c>
       <c r="K37" t="n">
-        <v>2749</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4025,7 +4025,7 @@
         <v>-1</v>
       </c>
       <c r="F38" s="83" t="n">
-        <v>26920</v>
+        <v>26921</v>
       </c>
       <c r="G38" s="83" t="n">
         <v>167020</v>
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>30000</v>
+        <v>7895</v>
       </c>
       <c r="K38" t="n">
-        <v>1500</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4067,7 +4067,7 @@
         <v>7816</v>
       </c>
       <c r="G39" s="83" t="n">
-        <v>65542</v>
+        <v>65543</v>
       </c>
       <c r="H39" s="82" t="n">
         <v>-0.88</v>
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K39" t="n">
-        <v>750</v>
+        <v>658</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>129999</v>
+        <v>34211</v>
       </c>
       <c r="K41" t="n">
-        <v>6499</v>
+        <v>5702</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4175,7 +4175,7 @@
         <v>3164</v>
       </c>
       <c r="D42" s="85" t="n">
-        <v>7291</v>
+        <v>7292</v>
       </c>
       <c r="E42" s="195" t="n">
         <v>-0.5660676534598215</v>
@@ -4184,7 +4184,7 @@
         <v>246020</v>
       </c>
       <c r="G42" s="85" t="n">
-        <v>222599</v>
+        <v>222600</v>
       </c>
       <c r="H42" s="195" t="n">
         <v>0.11</v>
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>35000</v>
+        <v>9211</v>
       </c>
       <c r="K42" t="n">
-        <v>1591</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4211,7 +4211,7 @@
         </is>
       </c>
       <c r="C43" s="83" t="n">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="D43" s="83" t="n">
         <v>2083</v>
@@ -4220,10 +4220,10 @@
         <v>-0.3805263983154294</v>
       </c>
       <c r="F43" s="83" t="n">
-        <v>59437</v>
+        <v>59438</v>
       </c>
       <c r="G43" s="83" t="n">
-        <v>64822</v>
+        <v>64823</v>
       </c>
       <c r="H43" s="82" t="n">
         <v>-0.08</v>
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K43" t="n">
-        <v>435</v>
+        <v>224</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4259,10 +4259,10 @@
         <v>-0.9349333333333334</v>
       </c>
       <c r="F44" s="83" t="n">
-        <v>284868</v>
+        <v>284869</v>
       </c>
       <c r="G44" s="83" t="n">
-        <v>310632</v>
+        <v>310633</v>
       </c>
       <c r="H44" s="82" t="n">
         <v>-0.08</v>
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>9000</v>
+        <v>2368</v>
       </c>
       <c r="K44" t="n">
-        <v>443</v>
+        <v>374</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="C45" s="83" t="n">
-        <v>6619</v>
+        <v>6620</v>
       </c>
       <c r="D45" s="83" t="n">
         <v>8333</v>
@@ -4298,7 +4298,7 @@
         <v>-0.2056012048339838</v>
       </c>
       <c r="F45" s="83" t="n">
-        <v>246367</v>
+        <v>246368</v>
       </c>
       <c r="G45" s="83" t="n">
         <v>234599</v>
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>39999</v>
+        <v>10526</v>
       </c>
       <c r="K45" t="n">
-        <v>1669</v>
+        <v>651</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4328,7 +4328,7 @@
         </is>
       </c>
       <c r="C46" s="83" t="n">
-        <v>5016</v>
+        <v>5017</v>
       </c>
       <c r="D46" s="83" t="n">
         <v>5208</v>
@@ -4337,10 +4337,10 @@
         <v>-0.03678399999999948</v>
       </c>
       <c r="F46" s="83" t="n">
-        <v>111469</v>
+        <v>111470</v>
       </c>
       <c r="G46" s="83" t="n">
-        <v>113343</v>
+        <v>113344</v>
       </c>
       <c r="H46" s="82" t="n">
         <v>-0.02</v>
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K46" t="n">
-        <v>999</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4376,10 +4376,10 @@
         <v>0.04559841918945629</v>
       </c>
       <c r="F47" s="83" t="n">
-        <v>47113</v>
+        <v>47114</v>
       </c>
       <c r="G47" s="83" t="n">
-        <v>42367</v>
+        <v>42368</v>
       </c>
       <c r="H47" s="82" t="n">
         <v>0.11</v>
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K47" t="n">
-        <v>391</v>
+        <v>76</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4454,7 +4454,7 @@
         <v>-0.194881103448275</v>
       </c>
       <c r="F49" s="80" t="n">
-        <v>1472552</v>
+        <v>1472553</v>
       </c>
       <c r="G49" s="80" t="n">
         <v>1382748</v>
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>144999</v>
+        <v>38158</v>
       </c>
       <c r="K49" t="n">
-        <v>6033</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4484,7 +4484,7 @@
         </is>
       </c>
       <c r="C50" s="85" t="n">
-        <v>9618</v>
+        <v>9619</v>
       </c>
       <c r="D50" s="85" t="n">
         <v>12500</v>
@@ -4493,10 +4493,10 @@
         <v>-0.2304832128906249</v>
       </c>
       <c r="F50" s="85" t="n">
-        <v>358177</v>
+        <v>358178</v>
       </c>
       <c r="G50" s="85" t="n">
-        <v>377716</v>
+        <v>377717</v>
       </c>
       <c r="H50" s="195" t="n">
         <v>-0.05</v>
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>60000</v>
+        <v>15789</v>
       </c>
       <c r="K50" t="n">
-        <v>2519</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="C51" s="83" t="n">
-        <v>2651</v>
+        <v>2652</v>
       </c>
       <c r="D51" s="83" t="n">
         <v>2708</v>
@@ -4532,10 +4532,10 @@
         <v>-0.02082215857872372</v>
       </c>
       <c r="F51" s="83" t="n">
-        <v>94963</v>
+        <v>94964</v>
       </c>
       <c r="G51" s="83" t="n">
-        <v>85505</v>
+        <v>85506</v>
       </c>
       <c r="H51" s="82" t="n">
         <v>0.11</v>
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>12999</v>
+        <v>3421</v>
       </c>
       <c r="K51" t="n">
-        <v>517</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="C52" s="83" t="n">
-        <v>2274</v>
+        <v>2275</v>
       </c>
       <c r="D52" s="83" t="n">
         <v>3125</v>
@@ -4571,10 +4571,10 @@
         <v>-0.2721023828124993</v>
       </c>
       <c r="F52" s="83" t="n">
-        <v>301582</v>
+        <v>301583</v>
       </c>
       <c r="G52" s="83" t="n">
-        <v>324739</v>
+        <v>324740</v>
       </c>
       <c r="H52" s="82" t="n">
         <v>-0.07000000000000001</v>
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K52" t="n">
-        <v>636</v>
+        <v>279</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4610,10 +4610,10 @@
         <v>-0.31694</v>
       </c>
       <c r="F53" s="83" t="n">
-        <v>364642</v>
+        <v>364643</v>
       </c>
       <c r="G53" s="83" t="n">
-        <v>330224</v>
+        <v>330225</v>
       </c>
       <c r="H53" s="82" t="n">
         <v>0.1</v>
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>60000</v>
+        <v>15789</v>
       </c>
       <c r="K53" t="n">
-        <v>2573</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>45000</v>
+        <v>11842</v>
       </c>
       <c r="K54" t="n">
-        <v>1971</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4679,7 +4679,7 @@
         </is>
       </c>
       <c r="C55" s="83" t="n">
-        <v>4290</v>
+        <v>4291</v>
       </c>
       <c r="D55" s="83" t="n">
         <v>5208</v>
@@ -4688,10 +4688,10 @@
         <v>-0.1761664257812489</v>
       </c>
       <c r="F55" s="83" t="n">
-        <v>127607</v>
+        <v>127608</v>
       </c>
       <c r="G55" s="83" t="n">
-        <v>94380</v>
+        <v>94381</v>
       </c>
       <c r="H55" s="82" t="n">
         <v>0.35</v>
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K55" t="n">
-        <v>1035</v>
+        <v>381</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4760,7 +4760,7 @@
         <v>47835</v>
       </c>
       <c r="D57" s="80" t="n">
-        <v>54166</v>
+        <v>54167</v>
       </c>
       <c r="E57" s="201" t="n">
         <v>-0.116885292307693</v>
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>260000</v>
+        <v>68421</v>
       </c>
       <c r="K57" t="n">
-        <v>10608</v>
+        <v>3431</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>45000</v>
+        <v>11842</v>
       </c>
       <c r="K58" t="n">
-        <v>2068</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4835,7 +4835,7 @@
         </is>
       </c>
       <c r="C59" s="83" t="n">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="D59" s="83" t="n">
         <v>2500</v>
@@ -4847,19 +4847,19 @@
         <v>54796</v>
       </c>
       <c r="G59" s="83" t="n">
-        <v>63686</v>
+        <v>63687</v>
       </c>
       <c r="H59" s="82" t="n">
         <v>-0.14</v>
       </c>
       <c r="I59" s="83" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K59" t="n">
-        <v>534</v>
+        <v>310</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4874,7 +4874,7 @@
         </is>
       </c>
       <c r="C60" s="83" t="n">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="D60" s="83" t="n">
         <v>3333</v>
@@ -4883,7 +4883,7 @@
         <v>-0.6793910030458981</v>
       </c>
       <c r="F60" s="83" t="n">
-        <v>363222</v>
+        <v>363223</v>
       </c>
       <c r="G60" s="83" t="n">
         <v>147092</v>
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>15999</v>
+        <v>4211</v>
       </c>
       <c r="K60" t="n">
-        <v>746</v>
+        <v>524</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4922,7 +4922,7 @@
         <v>-0.1863653997802738</v>
       </c>
       <c r="F61" s="83" t="n">
-        <v>296146</v>
+        <v>296147</v>
       </c>
       <c r="G61" s="83" t="n">
         <v>241715</v>
@@ -4931,13 +4931,13 @@
         <v>0.23</v>
       </c>
       <c r="I61" s="83" t="n">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>39999</v>
+        <v>10526</v>
       </c>
       <c r="K61" t="n">
-        <v>1660</v>
+        <v>624</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4961,7 +4961,7 @@
         <v>-0.03669999999999995</v>
       </c>
       <c r="F62" s="83" t="n">
-        <v>74658</v>
+        <v>74659</v>
       </c>
       <c r="G62" s="83" t="n">
         <v>71255</v>
@@ -4970,13 +4970,13 @@
         <v>0.05</v>
       </c>
       <c r="I62" s="83" t="n">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K62" t="n">
-        <v>479</v>
+        <v>125</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5003,7 +5003,7 @@
         <v>67242</v>
       </c>
       <c r="G63" s="83" t="n">
-        <v>55406</v>
+        <v>55407</v>
       </c>
       <c r="H63" s="82" t="n">
         <v>0.21</v>
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K63" t="n">
-        <v>433</v>
+        <v>216</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5072,7 +5072,7 @@
         <v>25930</v>
       </c>
       <c r="D65" s="80" t="n">
-        <v>35416</v>
+        <v>35417</v>
       </c>
       <c r="E65" s="201" t="n">
         <v>-0.2678515882117656</v>
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>170000</v>
+        <v>44737</v>
       </c>
       <c r="K65" t="n">
-        <v>7203</v>
+        <v>3134</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5120,7 +5120,7 @@
         <v>109274</v>
       </c>
       <c r="G66" s="85" t="n">
-        <v>135756</v>
+        <v>135757</v>
       </c>
       <c r="H66" s="195" t="n">
         <v>-0.2</v>
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K66" t="n">
-        <v>1249</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5159,7 +5159,7 @@
         <v>28539</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>36387</v>
+        <v>36388</v>
       </c>
       <c r="H67" s="82" t="n">
         <v>-0.22</v>
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K67" t="n">
-        <v>499</v>
+        <v>439</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K68" t="n">
-        <v>499</v>
+        <v>439</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5228,7 +5228,7 @@
         <v>0</v>
       </c>
       <c r="D69" s="83" t="n">
-        <v>7291</v>
+        <v>7292</v>
       </c>
       <c r="E69" s="82" t="n">
         <v>-1</v>
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>35000</v>
+        <v>9211</v>
       </c>
       <c r="K69" t="n">
-        <v>1750</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K70" t="n">
-        <v>600</v>
+        <v>526</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K71" t="n">
-        <v>1249</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5384,13 +5384,13 @@
         <v>0</v>
       </c>
       <c r="D73" s="80" t="n">
-        <v>29166</v>
+        <v>29167</v>
       </c>
       <c r="E73" s="201" t="n">
         <v>-1</v>
       </c>
       <c r="F73" s="80" t="n">
-        <v>782004</v>
+        <v>782005</v>
       </c>
       <c r="G73" s="80" t="n">
         <v>841660</v>
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>140000</v>
+        <v>36842</v>
       </c>
       <c r="K73" t="n">
-        <v>7000</v>
+        <v>6140</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5429,7 +5429,7 @@
         <v>-0.5448495115885416</v>
       </c>
       <c r="F74" s="85" t="n">
-        <v>305221</v>
+        <v>305222</v>
       </c>
       <c r="G74" s="85" t="n">
         <v>454660</v>
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>60000</v>
+        <v>15789</v>
       </c>
       <c r="K74" t="n">
-        <v>2715</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5468,10 +5468,10 @@
         <v>-0.4191926201453569</v>
       </c>
       <c r="F75" s="83" t="n">
-        <v>67408</v>
+        <v>67409</v>
       </c>
       <c r="G75" s="83" t="n">
-        <v>84387</v>
+        <v>84388</v>
       </c>
       <c r="H75" s="82" t="n">
         <v>-0.2</v>
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>12999</v>
+        <v>3421</v>
       </c>
       <c r="K75" t="n">
-        <v>571</v>
+        <v>308</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5498,7 +5498,7 @@
         </is>
       </c>
       <c r="C76" s="83" t="n">
-        <v>1983</v>
+        <v>1984</v>
       </c>
       <c r="D76" s="83" t="n">
         <v>6250</v>
@@ -5507,7 +5507,7 @@
         <v>-0.6826000036621087</v>
       </c>
       <c r="F76" s="83" t="n">
-        <v>208620</v>
+        <v>208621</v>
       </c>
       <c r="G76" s="83" t="n">
         <v>231794</v>
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>30000</v>
+        <v>7895</v>
       </c>
       <c r="K76" t="n">
-        <v>1400</v>
+        <v>985</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5555,13 +5555,13 @@
         </is>
       </c>
       <c r="I77" s="83" t="n">
-        <v>3781</v>
+        <v>3782</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>-425</v>
+        <v>-1419</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="250">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="E78" s="82" t="n"/>
       <c r="F78" s="83" t="n">
-        <v>63718</v>
+        <v>63719</v>
       </c>
       <c r="G78" s="83" t="n">
         <v>6474</v>
@@ -5592,13 +5592,13 @@
         <v>8.84</v>
       </c>
       <c r="I78" s="83" t="n">
-        <v>2991</v>
+        <v>2992</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>-242</v>
+        <v>-808</v>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="250">
@@ -5613,14 +5613,14 @@
         </is>
       </c>
       <c r="C79" s="83" t="n">
-        <v>2468</v>
+        <v>2469</v>
       </c>
       <c r="D79" s="83" t="n">
         <v>0</v>
       </c>
       <c r="E79" s="82" t="n"/>
       <c r="F79" s="83" t="n">
-        <v>21971</v>
+        <v>21972</v>
       </c>
       <c r="G79" s="83" t="n">
         <v>389</v>
@@ -5631,13 +5631,13 @@
         </is>
       </c>
       <c r="I79" s="83" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
       </c>
       <c r="K79" t="n">
-        <v>-123</v>
+        <v>-411</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="250">
@@ -5700,7 +5700,7 @@
         <v>0.1989448413333343</v>
       </c>
       <c r="F81" s="80" t="n">
-        <v>1357561</v>
+        <v>1357562</v>
       </c>
       <c r="G81" s="80" t="n">
         <v>1095971</v>
@@ -5709,13 +5709,13 @@
         <v>0.24</v>
       </c>
       <c r="I81" s="80" t="n">
-        <v>15732</v>
+        <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>150000</v>
+        <v>39474</v>
       </c>
       <c r="K81" t="n">
-        <v>5626</v>
+        <v>334</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5737,10 +5737,10 @@
       </c>
       <c r="E82" s="195" t="n"/>
       <c r="F82" s="85" t="n">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="G82" s="85" t="n">
-        <v>8508</v>
+        <v>8509</v>
       </c>
       <c r="H82" s="195" t="n">
         <v>-0.9</v>
@@ -5777,7 +5777,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="83" t="n">
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="H83" s="82" t="n">
         <v>-1</v>
@@ -5814,7 +5814,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="83" t="n">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="H84" s="82" t="n">
         <v>-1</v>
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>42999</v>
+        <v>11316</v>
       </c>
       <c r="K85" t="n">
-        <v>2149</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5883,7 +5883,7 @@
         <v>0</v>
       </c>
       <c r="D86" s="83" t="n">
-        <v>4791</v>
+        <v>4792</v>
       </c>
       <c r="E86" s="82" t="n">
         <v>-1</v>
@@ -5892,7 +5892,7 @@
         <v>15730</v>
       </c>
       <c r="G86" s="83" t="n">
-        <v>122006</v>
+        <v>122007</v>
       </c>
       <c r="H86" s="82" t="n">
         <v>-0.87</v>
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>23000</v>
+        <v>6053</v>
       </c>
       <c r="K86" t="n">
-        <v>1150</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5928,10 +5928,10 @@
         <v>-1</v>
       </c>
       <c r="F87" s="83" t="n">
-        <v>16724</v>
+        <v>16725</v>
       </c>
       <c r="G87" s="83" t="n">
-        <v>42952</v>
+        <v>42953</v>
       </c>
       <c r="H87" s="82" t="n">
         <v>-0.61</v>
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K87" t="n">
-        <v>600</v>
+        <v>526</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6006,7 +6006,7 @@
         <v>-1</v>
       </c>
       <c r="F89" s="80" t="n">
-        <v>184409</v>
+        <v>184410</v>
       </c>
       <c r="G89" s="80" t="n">
         <v>831747</v>
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>123000</v>
+        <v>32368</v>
       </c>
       <c r="K89" t="n">
-        <v>6150</v>
+        <v>5395</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6048,7 +6048,7 @@
         <v>321774</v>
       </c>
       <c r="G90" s="85" t="n">
-        <v>392981</v>
+        <v>392982</v>
       </c>
       <c r="H90" s="195" t="n">
         <v>-0.18</v>
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>69999</v>
+        <v>18421</v>
       </c>
       <c r="K90" t="n">
-        <v>3044</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6087,7 +6087,7 @@
         <v>83389</v>
       </c>
       <c r="G91" s="83" t="n">
-        <v>81416</v>
+        <v>81417</v>
       </c>
       <c r="H91" s="82" t="n">
         <v>0.02</v>
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K91" t="n">
-        <v>396</v>
+        <v>92</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="C92" s="83" t="n">
-        <v>3796</v>
+        <v>3797</v>
       </c>
       <c r="D92" s="83" t="n">
         <v>2500</v>
@@ -6123,10 +6123,10 @@
         <v>0.5186237200887041</v>
       </c>
       <c r="F92" s="83" t="n">
-        <v>149338</v>
+        <v>149339</v>
       </c>
       <c r="G92" s="83" t="n">
-        <v>343192</v>
+        <v>343193</v>
       </c>
       <c r="H92" s="82" t="n">
         <v>-0.5600000000000001</v>
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>12000</v>
+        <v>3158</v>
       </c>
       <c r="K92" t="n">
-        <v>410</v>
+        <v>-106</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="E95" s="82" t="n"/>
       <c r="F95" s="83" t="n">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="G95" s="83" t="n">
         <v>8497</v>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="C97" s="80" t="n">
-        <v>25387</v>
+        <v>25388</v>
       </c>
       <c r="D97" s="80" t="n">
         <v>31250</v>
@@ -6315,19 +6315,19 @@
         <v>947083</v>
       </c>
       <c r="G97" s="80" t="n">
-        <v>1286114</v>
+        <v>1286115</v>
       </c>
       <c r="H97" s="201" t="n">
         <v>-0.26</v>
       </c>
       <c r="I97" s="80" t="n">
-        <v>6325</v>
+        <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>150000</v>
+        <v>39474</v>
       </c>
       <c r="K97" t="n">
-        <v>6230</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6349,7 +6349,7 @@
       </c>
       <c r="E98" s="195" t="n"/>
       <c r="F98" s="85" t="n">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="G98" s="85" t="n">
         <v>19460</v>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="E99" s="82" t="n"/>
       <c r="F99" s="83" t="n">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="G99" s="83" t="n">
         <v>4053</v>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="E100" s="82" t="n"/>
       <c r="F100" s="83" t="n">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="G100" s="83" t="n">
         <v>2070</v>
@@ -6456,16 +6456,16 @@
         <v>10732</v>
       </c>
       <c r="D101" s="83" t="n">
-        <v>16666</v>
+        <v>16667</v>
       </c>
       <c r="E101" s="82" t="n">
         <v>-0.3560750011444109</v>
       </c>
       <c r="F101" s="83" t="n">
-        <v>418838</v>
+        <v>418839</v>
       </c>
       <c r="G101" s="83" t="n">
-        <v>461397</v>
+        <v>461398</v>
       </c>
       <c r="H101" s="82" t="n">
         <v>-0.09</v>
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>80000</v>
+        <v>21053</v>
       </c>
       <c r="K101" t="n">
-        <v>3463</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6504,19 +6504,19 @@
         <v>143725</v>
       </c>
       <c r="G102" s="83" t="n">
-        <v>187563</v>
+        <v>187564</v>
       </c>
       <c r="H102" s="82" t="n">
         <v>-0.23</v>
       </c>
       <c r="I102" s="83" t="n">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>39999</v>
+        <v>10526</v>
       </c>
       <c r="K102" t="n">
-        <v>1734</v>
+        <v>870</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6531,16 +6531,16 @@
         </is>
       </c>
       <c r="C103" s="83" t="n">
-        <v>8116</v>
+        <v>8117</v>
       </c>
       <c r="D103" s="83" t="n">
-        <v>5416</v>
+        <v>5417</v>
       </c>
       <c r="E103" s="82" t="n">
         <v>0.4985134241943356</v>
       </c>
       <c r="F103" s="83" t="n">
-        <v>115465</v>
+        <v>115466</v>
       </c>
       <c r="G103" s="83" t="n">
         <v>117988</v>
@@ -6549,13 +6549,13 @@
         <v>-0.02</v>
       </c>
       <c r="I103" s="83" t="n">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>26000</v>
+        <v>6842</v>
       </c>
       <c r="K103" t="n">
-        <v>894</v>
+        <v>-212</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6618,22 +6618,22 @@
         <v>-0.1015991333333333</v>
       </c>
       <c r="F105" s="80" t="n">
-        <v>1054158</v>
+        <v>1054159</v>
       </c>
       <c r="G105" s="80" t="n">
-        <v>1207116</v>
+        <v>1207117</v>
       </c>
       <c r="H105" s="201" t="n">
         <v>-0.13</v>
       </c>
       <c r="I105" s="80" t="n">
-        <v>9206</v>
+        <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>180000</v>
+        <v>47368</v>
       </c>
       <c r="K105" t="n">
-        <v>7315</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6655,10 +6655,10 @@
       </c>
       <c r="E106" s="195" t="n"/>
       <c r="F106" s="85" t="n">
-        <v>11887</v>
+        <v>11888</v>
       </c>
       <c r="G106" s="85" t="n">
-        <v>12827</v>
+        <v>12828</v>
       </c>
       <c r="H106" s="195" t="n">
         <v>-0.07000000000000001</v>
@@ -6692,10 +6692,10 @@
       </c>
       <c r="E107" s="82" t="n"/>
       <c r="F107" s="83" t="n">
-        <v>2167</v>
+        <v>2168</v>
       </c>
       <c r="G107" s="83" t="n">
-        <v>3458</v>
+        <v>3459</v>
       </c>
       <c r="H107" s="82" t="n">
         <v>-0.37</v>
@@ -6729,10 +6729,10 @@
       </c>
       <c r="E108" s="82" t="n"/>
       <c r="F108" s="83" t="n">
-        <v>3121</v>
+        <v>3122</v>
       </c>
       <c r="G108" s="83" t="n">
-        <v>4612</v>
+        <v>4613</v>
       </c>
       <c r="H108" s="82" t="n">
         <v>-0.32</v>
@@ -6759,10 +6759,10 @@
         </is>
       </c>
       <c r="C109" s="83" t="n">
-        <v>11195</v>
+        <v>11196</v>
       </c>
       <c r="D109" s="83" t="n">
-        <v>16666</v>
+        <v>16667</v>
       </c>
       <c r="E109" s="82" t="n">
         <v>-0.3282443966674817</v>
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>80000</v>
+        <v>21053</v>
       </c>
       <c r="K109" t="n">
-        <v>3440</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6807,22 +6807,22 @@
         <v>-0.08520924424913245</v>
       </c>
       <c r="F110" s="83" t="n">
-        <v>147994</v>
+        <v>147995</v>
       </c>
       <c r="G110" s="83" t="n">
-        <v>232101</v>
+        <v>232102</v>
       </c>
       <c r="H110" s="82" t="n">
         <v>-0.36</v>
       </c>
       <c r="I110" s="83" t="n">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>45000</v>
+        <v>11842</v>
       </c>
       <c r="K110" t="n">
-        <v>1821</v>
+        <v>544</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="C111" s="83" t="n">
-        <v>6710</v>
+        <v>6711</v>
       </c>
       <c r="D111" s="83" t="n">
         <v>5208</v>
@@ -6849,19 +6849,19 @@
         <v>90649</v>
       </c>
       <c r="G111" s="83" t="n">
-        <v>129723</v>
+        <v>129724</v>
       </c>
       <c r="H111" s="82" t="n">
         <v>-0.3</v>
       </c>
       <c r="I111" s="83" t="n">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K111" t="n">
-        <v>914</v>
+        <v>-22</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6924,22 +6924,22 @@
         <v>0.09198613333333339</v>
       </c>
       <c r="F113" s="80" t="n">
-        <v>1004184</v>
+        <v>1004185</v>
       </c>
       <c r="G113" s="80" t="n">
-        <v>1346018</v>
+        <v>1346019</v>
       </c>
       <c r="H113" s="201" t="n">
         <v>-0.25</v>
       </c>
       <c r="I113" s="80" t="n">
-        <v>5379</v>
+        <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>180000</v>
+        <v>47368</v>
       </c>
       <c r="K113" t="n">
-        <v>6952</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6954,10 +6954,10 @@
         </is>
       </c>
       <c r="C114" s="85" t="n">
-        <v>16658</v>
+        <v>16659</v>
       </c>
       <c r="D114" s="85" t="n">
-        <v>13541</v>
+        <v>13542</v>
       </c>
       <c r="E114" s="195" t="n">
         <v>0.2302010094711522</v>
@@ -6972,13 +6972,13 @@
         <v>-0.28</v>
       </c>
       <c r="I114" s="85" t="n">
-        <v>3029</v>
+        <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>65000</v>
+        <v>17105</v>
       </c>
       <c r="K114" t="n">
-        <v>2417</v>
+        <v>74</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -6996,28 +6996,28 @@
         <v>2702</v>
       </c>
       <c r="D115" s="83" t="n">
-        <v>4166</v>
+        <v>4167</v>
       </c>
       <c r="E115" s="82" t="n">
         <v>-0.3514216046142572</v>
       </c>
       <c r="F115" s="83" t="n">
-        <v>85661</v>
+        <v>85662</v>
       </c>
       <c r="G115" s="83" t="n">
-        <v>92139</v>
+        <v>92140</v>
       </c>
       <c r="H115" s="82" t="n">
         <v>-0.07000000000000001</v>
       </c>
       <c r="I115" s="83" t="n">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>20000</v>
+        <v>5263</v>
       </c>
       <c r="K115" t="n">
-        <v>864</v>
+        <v>427</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7032,7 +7032,7 @@
         </is>
       </c>
       <c r="C116" s="83" t="n">
-        <v>4621</v>
+        <v>4622</v>
       </c>
       <c r="D116" s="83" t="n">
         <v>5208</v>
@@ -7044,7 +7044,7 @@
         <v>187402</v>
       </c>
       <c r="G116" s="83" t="n">
-        <v>311638</v>
+        <v>311639</v>
       </c>
       <c r="H116" s="82" t="n">
         <v>-0.4</v>
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K116" t="n">
-        <v>1018</v>
+        <v>326</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="E117" s="82" t="n"/>
       <c r="F117" s="83" t="n">
-        <v>5694</v>
+        <v>5695</v>
       </c>
       <c r="G117" s="83" t="n">
         <v>0</v>
@@ -7156,7 +7156,7 @@
       </c>
       <c r="E119" s="82" t="n"/>
       <c r="F119" s="83" t="n">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G119" s="83" t="n">
         <v>0</v>
@@ -7236,22 +7236,22 @@
         <v>0.18832129864</v>
       </c>
       <c r="F121" s="80" t="n">
-        <v>949436</v>
+        <v>949437</v>
       </c>
       <c r="G121" s="80" t="n">
-        <v>1224621</v>
+        <v>1224622</v>
       </c>
       <c r="H121" s="201" t="n">
         <v>-0.22</v>
       </c>
       <c r="I121" s="80" t="n">
-        <v>6772</v>
+        <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>150000</v>
+        <v>39474</v>
       </c>
       <c r="K121" t="n">
-        <v>5643</v>
+        <v>390</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7269,16 +7269,16 @@
         <v>11369</v>
       </c>
       <c r="D122" s="85" t="n">
-        <v>14166</v>
+        <v>14167</v>
       </c>
       <c r="E122" s="195" t="n">
         <v>-0.1974795180376866</v>
       </c>
       <c r="F122" s="85" t="n">
-        <v>351718</v>
+        <v>351719</v>
       </c>
       <c r="G122" s="85" t="n">
-        <v>462869</v>
+        <v>462870</v>
       </c>
       <c r="H122" s="195" t="n">
         <v>-0.24</v>
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>68000</v>
+        <v>17895</v>
       </c>
       <c r="K122" t="n">
-        <v>2831</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7305,7 +7305,7 @@
         </is>
       </c>
       <c r="C123" s="83" t="n">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="D123" s="83" t="n">
         <v>3125</v>
@@ -7314,7 +7314,7 @@
         <v>-0.6160256005859359</v>
       </c>
       <c r="F123" s="83" t="n">
-        <v>69735</v>
+        <v>69736</v>
       </c>
       <c r="G123" s="83" t="n">
         <v>84387</v>
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K123" t="n">
-        <v>690</v>
+        <v>458</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7344,7 +7344,7 @@
         </is>
       </c>
       <c r="C124" s="83" t="n">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="D124" s="83" t="n">
         <v>2083</v>
@@ -7353,7 +7353,7 @@
         <v>-0.4879936026000967</v>
       </c>
       <c r="F124" s="83" t="n">
-        <v>275085</v>
+        <v>275086</v>
       </c>
       <c r="G124" s="83" t="n">
         <v>225743</v>
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K124" t="n">
-        <v>446</v>
+        <v>261</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="C125" s="83" t="n">
-        <v>12764</v>
+        <v>12765</v>
       </c>
       <c r="D125" s="83" t="n">
         <v>15625</v>
@@ -7392,10 +7392,10 @@
         <v>-0.1830611201171904</v>
       </c>
       <c r="F125" s="83" t="n">
-        <v>348871</v>
+        <v>348872</v>
       </c>
       <c r="G125" s="83" t="n">
-        <v>432907</v>
+        <v>432908</v>
       </c>
       <c r="H125" s="82" t="n">
         <v>-0.19</v>
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>75000</v>
+        <v>19737</v>
       </c>
       <c r="K125" t="n">
-        <v>3111</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7425,16 +7425,16 @@
         <v>11009</v>
       </c>
       <c r="D126" s="83" t="n">
-        <v>6666</v>
+        <v>6667</v>
       </c>
       <c r="E126" s="82" t="n">
         <v>0.6513499999999992</v>
       </c>
       <c r="F126" s="83" t="n">
-        <v>148481</v>
+        <v>148482</v>
       </c>
       <c r="G126" s="83" t="n">
-        <v>154142</v>
+        <v>154143</v>
       </c>
       <c r="H126" s="82" t="n">
         <v>-0.04</v>
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>32000</v>
+        <v>8421</v>
       </c>
       <c r="K126" t="n">
-        <v>1049</v>
+        <v>-431</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7461,7 +7461,7 @@
         </is>
       </c>
       <c r="C127" s="83" t="n">
-        <v>2085</v>
+        <v>2086</v>
       </c>
       <c r="D127" s="83" t="n">
         <v>2083</v>
@@ -7470,10 +7470,10 @@
         <v>0.00106880615234406</v>
       </c>
       <c r="F127" s="83" t="n">
-        <v>63197</v>
+        <v>63198</v>
       </c>
       <c r="G127" s="83" t="n">
-        <v>28932</v>
+        <v>28933</v>
       </c>
       <c r="H127" s="82" t="n">
         <v>1.18</v>
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K127" t="n">
-        <v>395</v>
+        <v>91</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7548,7 +7548,7 @@
         <v>-0.06617491428571376</v>
       </c>
       <c r="F129" s="80" t="n">
-        <v>1842830</v>
+        <v>1842831</v>
       </c>
       <c r="G129" s="80" t="n">
         <v>1967384</v>
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>279999</v>
+        <v>73684</v>
       </c>
       <c r="K129" t="n">
-        <v>11276</v>
+        <v>3202</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7578,16 +7578,16 @@
         </is>
       </c>
       <c r="C130" s="85" t="n">
-        <v>6179</v>
+        <v>6180</v>
       </c>
       <c r="D130" s="85" t="n">
-        <v>4166</v>
+        <v>4167</v>
       </c>
       <c r="E130" s="195" t="n">
         <v>0.4831495800781245</v>
       </c>
       <c r="F130" s="85" t="n">
-        <v>141180</v>
+        <v>141181</v>
       </c>
       <c r="G130" s="85" t="n">
         <v>0</v>
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>20000</v>
+        <v>5263</v>
       </c>
       <c r="K130" t="n">
-        <v>691</v>
+        <v>-153</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7619,7 +7619,7 @@
         </is>
       </c>
       <c r="C131" s="83" t="n">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="D131" s="83" t="n">
         <v>2083</v>
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K131" t="n">
-        <v>447</v>
+        <v>264</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7660,7 +7660,7 @@
         </is>
       </c>
       <c r="C132" s="83" t="n">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="D132" s="83" t="n">
         <v>2083</v>
@@ -7669,7 +7669,7 @@
         <v>-0.4812015881347639</v>
       </c>
       <c r="F132" s="83" t="n">
-        <v>146027</v>
+        <v>146028</v>
       </c>
       <c r="G132" s="83" t="n">
         <v>0</v>
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K132" t="n">
-        <v>445</v>
+        <v>258</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7710,7 +7710,7 @@
         <v>0.08678720776367244</v>
       </c>
       <c r="F133" s="83" t="n">
-        <v>165040</v>
+        <v>165041</v>
       </c>
       <c r="G133" s="83" t="n">
         <v>0</v>
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>24999</v>
+        <v>6579</v>
       </c>
       <c r="K133" t="n">
-        <v>966</v>
+        <v>153</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7751,7 +7751,7 @@
         <v>0.3780255957031264</v>
       </c>
       <c r="F134" s="83" t="n">
-        <v>60579</v>
+        <v>60580</v>
       </c>
       <c r="G134" s="83" t="n">
         <v>0</v>
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K134" t="n">
-        <v>534</v>
+        <v>-60</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7783,7 +7783,7 @@
         </is>
       </c>
       <c r="C135" s="83" t="n">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="D135" s="83" t="n">
         <v>2083</v>
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K135" t="n">
-        <v>398</v>
+        <v>100</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7863,10 +7863,10 @@
         </is>
       </c>
       <c r="C137" s="80" t="n">
-        <v>32935</v>
+        <v>32936</v>
       </c>
       <c r="D137" s="80" t="n">
-        <v>29166</v>
+        <v>29167</v>
       </c>
       <c r="E137" s="201" t="n">
         <v>0.12923257142857</v>
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>140000</v>
+        <v>36842</v>
       </c>
       <c r="K137" t="n">
-        <v>5353</v>
+        <v>651</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7904,10 +7904,10 @@
         </is>
       </c>
       <c r="C138" s="85" t="n">
-        <v>6160</v>
+        <v>6161</v>
       </c>
       <c r="D138" s="85" t="n">
-        <v>4166</v>
+        <v>4167</v>
       </c>
       <c r="E138" s="195" t="n">
         <v>0.478534414062499</v>
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>20000</v>
+        <v>5263</v>
       </c>
       <c r="K138" t="n">
-        <v>691</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7952,7 +7952,7 @@
         <v>-0.3998319961547863</v>
       </c>
       <c r="F139" s="83" t="n">
-        <v>48621</v>
+        <v>48622</v>
       </c>
       <c r="G139" s="83" t="n">
         <v>77247</v>
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K139" t="n">
-        <v>437</v>
+        <v>230</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K140" t="n">
-        <v>488</v>
+        <v>400</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8033,7 +8033,7 @@
         <v>224058</v>
       </c>
       <c r="G141" s="83" t="n">
-        <v>392991</v>
+        <v>392992</v>
       </c>
       <c r="H141" s="82" t="n">
         <v>-0.43</v>
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>30000</v>
+        <v>7895</v>
       </c>
       <c r="K141" t="n">
-        <v>1162</v>
+        <v>190</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8069,7 +8069,7 @@
         <v>-0.13152</v>
       </c>
       <c r="F142" s="83" t="n">
-        <v>43275</v>
+        <v>43276</v>
       </c>
       <c r="G142" s="83" t="n">
         <v>136218</v>
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K142" t="n">
-        <v>614</v>
+        <v>206</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8099,7 +8099,7 @@
         </is>
       </c>
       <c r="C143" s="83" t="n">
-        <v>1753</v>
+        <v>1754</v>
       </c>
       <c r="D143" s="83" t="n">
         <v>3125</v>
@@ -8108,10 +8108,10 @@
         <v>-0.4387744140624992</v>
       </c>
       <c r="F143" s="83" t="n">
-        <v>45800</v>
+        <v>45801</v>
       </c>
       <c r="G143" s="83" t="n">
-        <v>99397</v>
+        <v>99398</v>
       </c>
       <c r="H143" s="82" t="n">
         <v>-0.54</v>
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K143" t="n">
-        <v>662</v>
+        <v>366</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8177,7 +8177,7 @@
         </is>
       </c>
       <c r="C145" s="80" t="n">
-        <v>26940</v>
+        <v>26941</v>
       </c>
       <c r="D145" s="80" t="n">
         <v>31250</v>
@@ -8186,10 +8186,10 @@
         <v>-0.1378902399999999</v>
       </c>
       <c r="F145" s="80" t="n">
-        <v>1134536</v>
+        <v>1134537</v>
       </c>
       <c r="G145" s="80" t="n">
-        <v>2143278</v>
+        <v>2143279</v>
       </c>
       <c r="H145" s="201" t="n">
         <v>-0.47</v>
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>150000</v>
+        <v>39474</v>
       </c>
       <c r="K145" t="n">
-        <v>6152</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8216,19 +8216,19 @@
         </is>
       </c>
       <c r="C146" s="85" t="n">
-        <v>6307</v>
+        <v>6308</v>
       </c>
       <c r="D146" s="85" t="n">
-        <v>7291</v>
+        <v>7292</v>
       </c>
       <c r="E146" s="195" t="n">
         <v>-0.1349316517857146</v>
       </c>
       <c r="F146" s="85" t="n">
-        <v>198149</v>
+        <v>198150</v>
       </c>
       <c r="G146" s="85" t="n">
-        <v>269026</v>
+        <v>269027</v>
       </c>
       <c r="H146" s="195" t="n">
         <v>-0.26</v>
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>35000</v>
+        <v>9211</v>
       </c>
       <c r="K146" t="n">
-        <v>1434</v>
+        <v>484</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K147" t="n">
-        <v>456</v>
+        <v>294</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>12500</v>
+        <v>3289</v>
       </c>
       <c r="K148" t="n">
-        <v>573</v>
+        <v>375</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8342,7 +8342,7 @@
         <v>-0.04106678710937406</v>
       </c>
       <c r="F149" s="83" t="n">
-        <v>168543</v>
+        <v>168544</v>
       </c>
       <c r="G149" s="83" t="n">
         <v>180942</v>
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>39999</v>
+        <v>10526</v>
       </c>
       <c r="K149" t="n">
-        <v>1600</v>
+        <v>423</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8372,10 +8372,10 @@
         </is>
       </c>
       <c r="C150" s="83" t="n">
-        <v>4653</v>
+        <v>4654</v>
       </c>
       <c r="D150" s="83" t="n">
-        <v>4166</v>
+        <v>4167</v>
       </c>
       <c r="E150" s="82" t="n">
         <v>0.1168999999999991</v>
@@ -8384,7 +8384,7 @@
         <v>61262</v>
       </c>
       <c r="G150" s="83" t="n">
-        <v>78351</v>
+        <v>78352</v>
       </c>
       <c r="H150" s="82" t="n">
         <v>-0.22</v>
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>20000</v>
+        <v>5263</v>
       </c>
       <c r="K150" t="n">
-        <v>767</v>
+        <v>102</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8411,7 +8411,7 @@
         </is>
       </c>
       <c r="C151" s="83" t="n">
-        <v>3297</v>
+        <v>3298</v>
       </c>
       <c r="D151" s="83" t="n">
         <v>3125</v>
@@ -8420,10 +8420,10 @@
         <v>0.05535360839843828</v>
       </c>
       <c r="F151" s="83" t="n">
-        <v>31313</v>
+        <v>31314</v>
       </c>
       <c r="G151" s="83" t="n">
-        <v>57371</v>
+        <v>57372</v>
       </c>
       <c r="H151" s="82" t="n">
         <v>-0.45</v>
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>15000</v>
+        <v>3947</v>
       </c>
       <c r="K151" t="n">
-        <v>585</v>
+        <v>108</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8498,10 +8498,10 @@
         <v>0.06500287999999999</v>
       </c>
       <c r="F153" s="80" t="n">
-        <v>1018075</v>
+        <v>1018076</v>
       </c>
       <c r="G153" s="80" t="n">
-        <v>1167858</v>
+        <v>1167859</v>
       </c>
       <c r="H153" s="201" t="n">
         <v>-0.13</v>
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>150000</v>
+        <v>39474</v>
       </c>
       <c r="K153" t="n">
-        <v>5835</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8528,7 +8528,7 @@
         </is>
       </c>
       <c r="C154" s="85" t="n">
-        <v>5992</v>
+        <v>5993</v>
       </c>
       <c r="D154" s="85" t="n">
         <v>6250</v>
@@ -8537,7 +8537,7 @@
         <v>-0.04112491809895846</v>
       </c>
       <c r="F154" s="85" t="n">
-        <v>218796</v>
+        <v>218797</v>
       </c>
       <c r="G154" s="85" t="n">
         <v>243869</v>
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>30000</v>
+        <v>7895</v>
       </c>
       <c r="K154" t="n">
-        <v>1200</v>
+        <v>317</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8579,19 +8579,19 @@
         <v>52889</v>
       </c>
       <c r="G155" s="83" t="n">
-        <v>56497</v>
+        <v>56498</v>
       </c>
       <c r="H155" s="82" t="n">
         <v>-0.06</v>
       </c>
       <c r="I155" s="83" t="n">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K155" t="n">
-        <v>401</v>
+        <v>109</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8606,7 +8606,7 @@
         </is>
       </c>
       <c r="C156" s="83" t="n">
-        <v>2207</v>
+        <v>2208</v>
       </c>
       <c r="D156" s="83" t="n">
         <v>2083</v>
@@ -8618,19 +8618,19 @@
         <v>161815</v>
       </c>
       <c r="G156" s="83" t="n">
-        <v>131655</v>
+        <v>131656</v>
       </c>
       <c r="H156" s="82" t="n">
         <v>0.23</v>
       </c>
       <c r="I156" s="83" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>9999</v>
+        <v>2632</v>
       </c>
       <c r="K156" t="n">
-        <v>389</v>
+        <v>71</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8645,7 +8645,7 @@
         </is>
       </c>
       <c r="C157" s="83" t="n">
-        <v>6955</v>
+        <v>6956</v>
       </c>
       <c r="D157" s="83" t="n">
         <v>0</v>
@@ -8669,7 +8669,7 @@
         <v>0</v>
       </c>
       <c r="K157" t="n">
-        <v>-347</v>
+        <v>-1159</v>
       </c>
     </row>
     <row r="158" ht="14.25" customHeight="1" s="250">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="E158" s="82" t="n"/>
       <c r="F158" s="83" t="n">
-        <v>3209</v>
+        <v>3210</v>
       </c>
       <c r="G158" s="83" t="n">
         <v>0</v>
@@ -8702,13 +8702,13 @@
         </is>
       </c>
       <c r="I158" s="83" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J158" t="n">
         <v>0</v>
       </c>
       <c r="K158" t="n">
-        <v>-171</v>
+        <v>-570</v>
       </c>
     </row>
     <row r="159" ht="14.25" customHeight="1" s="250">
@@ -8730,7 +8730,7 @@
       </c>
       <c r="E159" s="82" t="n"/>
       <c r="F159" s="83" t="n">
-        <v>2184</v>
+        <v>2185</v>
       </c>
       <c r="G159" s="83" t="n">
         <v>0</v>
@@ -8741,13 +8741,13 @@
         </is>
       </c>
       <c r="I159" s="83" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J159" t="n">
         <v>0</v>
       </c>
       <c r="K159" t="n">
-        <v>-123</v>
+        <v>-413</v>
       </c>
     </row>
     <row r="160" ht="14.25" customHeight="1" s="250">
@@ -8801,7 +8801,7 @@
         </is>
       </c>
       <c r="C161" s="89" t="n">
-        <v>36802</v>
+        <v>36803</v>
       </c>
       <c r="D161" s="89" t="n">
         <v>25000</v>
@@ -8810,10 +8810,10 @@
         <v>0.4721043166666665</v>
       </c>
       <c r="F161" s="89" t="n">
-        <v>722394</v>
+        <v>722395</v>
       </c>
       <c r="G161" s="89" t="n">
-        <v>686239</v>
+        <v>686240</v>
       </c>
       <c r="H161" s="79" t="n">
         <v>0.05</v>
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>120000</v>
+        <v>31579</v>
       </c>
       <c r="K161" t="n">
-        <v>4159</v>
+        <v>-871</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="E162" s="79" t="n"/>
       <c r="F162" s="89" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="G162" s="89" t="n">
         <v>16065</v>
@@ -8887,7 +8887,7 @@
         <v>383</v>
       </c>
       <c r="G163" s="89" t="n">
-        <v>3962</v>
+        <v>3963</v>
       </c>
       <c r="H163" s="79" t="n">
         <v>-0.9</v>
@@ -8921,7 +8921,7 @@
       </c>
       <c r="E164" s="79" t="n"/>
       <c r="F164" s="89" t="n">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="G164" s="89" t="n">
         <v>20248</v>
@@ -8954,7 +8954,7 @@
         <v>0</v>
       </c>
       <c r="D165" s="89" t="n">
-        <v>13541</v>
+        <v>13542</v>
       </c>
       <c r="E165" s="79" t="n">
         <v>-1</v>
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>65000</v>
+        <v>17105</v>
       </c>
       <c r="K165" t="n">
-        <v>3250</v>
+        <v>2851</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -8993,13 +8993,13 @@
         <v>0</v>
       </c>
       <c r="D166" s="89" t="n">
-        <v>7916</v>
+        <v>7917</v>
       </c>
       <c r="E166" s="79" t="n">
         <v>-1</v>
       </c>
       <c r="F166" s="89" t="n">
-        <v>181761</v>
+        <v>181762</v>
       </c>
       <c r="G166" s="89" t="n">
         <v>219907</v>
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>38000</v>
+        <v>10000</v>
       </c>
       <c r="K166" t="n">
-        <v>1900</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9041,7 +9041,7 @@
         <v>156014</v>
       </c>
       <c r="G167" s="89" t="n">
-        <v>156148</v>
+        <v>156149</v>
       </c>
       <c r="H167" s="79" t="n">
         <v>0</v>
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>27999</v>
+        <v>7368</v>
       </c>
       <c r="K167" t="n">
-        <v>1399</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9110,7 +9110,7 @@
         <v>0</v>
       </c>
       <c r="D169" s="89" t="n">
-        <v>34791</v>
+        <v>34792</v>
       </c>
       <c r="E169" s="79" t="n">
         <v>-1</v>
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>167000</v>
+        <v>43947</v>
       </c>
       <c r="K169" t="n">
-        <v>8350</v>
+        <v>7325</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9146,7 +9146,7 @@
         </is>
       </c>
       <c r="C170" s="89" t="n">
-        <v>20051</v>
+        <v>20052</v>
       </c>
       <c r="D170" s="209" t="n">
         <v>155208</v>
@@ -9155,7 +9155,7 @@
         <v>-0.8708059536739408</v>
       </c>
       <c r="F170" s="89" t="n">
-        <v>13381000</v>
+        <v>13381001</v>
       </c>
       <c r="G170" s="89" t="n">
         <v>13643995</v>
@@ -9164,13 +9164,13 @@
         <v>-0.02</v>
       </c>
       <c r="I170" s="89" t="n">
-        <v>6509</v>
+        <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>744999</v>
+        <v>196053</v>
       </c>
       <c r="K170" t="n">
-        <v>36247</v>
+        <v>29333</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9185,7 +9185,7 @@
         </is>
       </c>
       <c r="C171" s="89" t="n">
-        <v>32784</v>
+        <v>32785</v>
       </c>
       <c r="D171" s="209" t="n">
         <v>37500</v>
@@ -9194,22 +9194,22 @@
         <v>-0.1257460199679918</v>
       </c>
       <c r="F171" s="89" t="n">
-        <v>3110091</v>
+        <v>3110092</v>
       </c>
       <c r="G171" s="89" t="n">
-        <v>3619339</v>
+        <v>3619340</v>
       </c>
       <c r="H171" s="79" t="n">
         <v>-0.14</v>
       </c>
       <c r="I171" s="89" t="n">
-        <v>12898</v>
+        <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>180000</v>
+        <v>47368</v>
       </c>
       <c r="K171" t="n">
-        <v>7360</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9224,7 +9224,7 @@
         </is>
       </c>
       <c r="C172" s="89" t="n">
-        <v>2613</v>
+        <v>2614</v>
       </c>
       <c r="D172" s="89" t="n">
         <v>28125</v>
@@ -9236,19 +9236,19 @@
         <v>4878021</v>
       </c>
       <c r="G172" s="89" t="n">
-        <v>6146767</v>
+        <v>6146768</v>
       </c>
       <c r="H172" s="79" t="n">
         <v>-0.21</v>
       </c>
       <c r="I172" s="89" t="n">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>135000</v>
+        <v>35526</v>
       </c>
       <c r="K172" t="n">
-        <v>6619</v>
+        <v>5485</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9263,10 +9263,10 @@
         </is>
       </c>
       <c r="C173" s="89" t="n">
-        <v>34770</v>
+        <v>34771</v>
       </c>
       <c r="D173" s="89" t="n">
-        <v>385416</v>
+        <v>385417</v>
       </c>
       <c r="E173" s="79" t="n">
         <v>-0.9097844639983635</v>
@@ -9275,7 +9275,7 @@
         <v>10930776</v>
       </c>
       <c r="G173" s="89" t="n">
-        <v>12177318</v>
+        <v>12177319</v>
       </c>
       <c r="H173" s="79" t="n">
         <v>-0.1</v>
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>1850000</v>
+        <v>486842</v>
       </c>
       <c r="K173" t="n">
-        <v>90761</v>
+        <v>75345</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9305,28 +9305,28 @@
         <v>15768</v>
       </c>
       <c r="D174" s="89" t="n">
-        <v>19791</v>
+        <v>19792</v>
       </c>
       <c r="E174" s="79" t="n">
         <v>-0.2032870200452308</v>
       </c>
       <c r="F174" s="89" t="n">
-        <v>692175</v>
+        <v>692176</v>
       </c>
       <c r="G174" s="89" t="n">
-        <v>1260547</v>
+        <v>1260548</v>
       </c>
       <c r="H174" s="79" t="n">
         <v>-0.45</v>
       </c>
       <c r="I174" s="89" t="n">
-        <v>3800</v>
+        <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>95000</v>
+        <v>25000</v>
       </c>
       <c r="K174" t="n">
-        <v>3961</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9341,10 +9341,10 @@
         </is>
       </c>
       <c r="C175" s="89" t="n">
-        <v>5595</v>
+        <v>5596</v>
       </c>
       <c r="D175" s="89" t="n">
-        <v>19791</v>
+        <v>19792</v>
       </c>
       <c r="E175" s="79" t="n">
         <v>-0.717259626302714</v>
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>95000</v>
+        <v>25000</v>
       </c>
       <c r="K175" t="n">
-        <v>4470</v>
+        <v>3234</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9419,7 +9419,7 @@
         </is>
       </c>
       <c r="C177" s="89" t="n">
-        <v>250392</v>
+        <v>250393</v>
       </c>
       <c r="D177" s="89" t="n">
         <v>887500</v>
@@ -9428,7 +9428,7 @@
         <v>-0.717867572161502</v>
       </c>
       <c r="F177" s="89" t="n">
-        <v>54594079</v>
+        <v>54594080</v>
       </c>
       <c r="G177" s="89" t="n">
         <v>57297099</v>
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>4260000</v>
+        <v>1121053</v>
       </c>
       <c r="K177" t="n">
-        <v>200480</v>
+        <v>145110</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9461,13 +9461,13 @@
         <v>41941</v>
       </c>
       <c r="D178" s="89" t="n">
-        <v>66666</v>
+        <v>66667</v>
       </c>
       <c r="E178" s="79" t="n">
         <v>-0.3708840024407953</v>
       </c>
       <c r="F178" s="89" t="n">
-        <v>1884107</v>
+        <v>1884108</v>
       </c>
       <c r="G178" s="89" t="n">
         <v>2155766</v>
@@ -9476,13 +9476,13 @@
         <v>-0.13</v>
       </c>
       <c r="I178" s="89" t="n">
-        <v>10388</v>
+        <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>320000</v>
+        <v>84211</v>
       </c>
       <c r="K178" t="n">
-        <v>13902</v>
+        <v>7045</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9500,7 +9500,7 @@
         <v>10940</v>
       </c>
       <c r="D179" s="89" t="n">
-        <v>16666</v>
+        <v>16667</v>
       </c>
       <c r="E179" s="79" t="n">
         <v>-0.3435786020278944</v>
@@ -9509,19 +9509,19 @@
         <v>416131</v>
       </c>
       <c r="G179" s="89" t="n">
-        <v>462663</v>
+        <v>462664</v>
       </c>
       <c r="H179" s="79" t="n">
         <v>-0.1</v>
       </c>
       <c r="I179" s="89" t="n">
-        <v>2167</v>
+        <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>80000</v>
+        <v>21053</v>
       </c>
       <c r="K179" t="n">
-        <v>3452</v>
+        <v>1685</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9536,16 +9536,16 @@
         </is>
       </c>
       <c r="C180" s="89" t="n">
-        <v>8658</v>
+        <v>8659</v>
       </c>
       <c r="D180" s="89" t="n">
-        <v>24166</v>
+        <v>24167</v>
       </c>
       <c r="E180" s="79" t="n">
         <v>-0.641716329555319</v>
       </c>
       <c r="F180" s="89" t="n">
-        <v>1755179</v>
+        <v>1755180</v>
       </c>
       <c r="G180" s="89" t="n">
         <v>1511826</v>
@@ -9554,13 +9554,13 @@
         <v>0.16</v>
       </c>
       <c r="I180" s="89" t="n">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>116000</v>
+        <v>30526</v>
       </c>
       <c r="K180" t="n">
-        <v>5367</v>
+        <v>3645</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9584,22 +9584,22 @@
         <v>-0.2084048556297826</v>
       </c>
       <c r="F181" s="89" t="n">
-        <v>2033754</v>
+        <v>2033755</v>
       </c>
       <c r="G181" s="89" t="n">
-        <v>1981135</v>
+        <v>1981136</v>
       </c>
       <c r="H181" s="79" t="n">
         <v>0.03</v>
       </c>
       <c r="I181" s="89" t="n">
-        <v>11858</v>
+        <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>318000</v>
+        <v>83684</v>
       </c>
       <c r="K181" t="n">
-        <v>13277</v>
+        <v>5207</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9614,10 +9614,10 @@
         </is>
       </c>
       <c r="C182" s="89" t="n">
-        <v>30943</v>
+        <v>30944</v>
       </c>
       <c r="D182" s="89" t="n">
-        <v>37916</v>
+        <v>37917</v>
       </c>
       <c r="E182" s="79" t="n">
         <v>-0.1839065498519726</v>
@@ -9626,7 +9626,7 @@
         <v>694522</v>
       </c>
       <c r="G182" s="89" t="n">
-        <v>813316</v>
+        <v>813317</v>
       </c>
       <c r="H182" s="79" t="n">
         <v>-0.15</v>
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>182000</v>
+        <v>47895</v>
       </c>
       <c r="K182" t="n">
-        <v>7552</v>
+        <v>2825</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9653,7 +9653,7 @@
         </is>
       </c>
       <c r="C183" s="89" t="n">
-        <v>17901</v>
+        <v>17902</v>
       </c>
       <c r="D183" s="89" t="n">
         <v>22708</v>
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>108999</v>
+        <v>28684</v>
       </c>
       <c r="K183" t="n">
-        <v>4554</v>
+        <v>1797</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9740,7 +9740,7 @@
         <v>-0.2440323312729666</v>
       </c>
       <c r="F185" s="89" t="n">
-        <v>10729242</v>
+        <v>10729243</v>
       </c>
       <c r="G185" s="89" t="n">
         <v>10693478</v>
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>1512999</v>
+        <v>398158</v>
       </c>
       <c r="K185" t="n">
-        <v>63735</v>
+        <v>26645</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9818,7 +9818,7 @@
         <v>-0.4772411094392471</v>
       </c>
       <c r="F187" s="89" t="n">
-        <v>75946677</v>
+        <v>75946678</v>
       </c>
       <c r="G187" s="89" t="n">
         <v>80227121</v>
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>7440000</v>
+        <v>1957895</v>
       </c>
       <c r="K187" t="n">
-        <v>331486</v>
+        <v>191270</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9857,10 +9857,10 @@
         <v>-0.5723919866666667</v>
       </c>
       <c r="F188" s="89" t="n">
-        <v>44414739</v>
+        <v>44414740</v>
       </c>
       <c r="G188" s="89" t="n">
-        <v>46516997</v>
+        <v>46516998</v>
       </c>
       <c r="H188" s="79" t="n">
         <v>-0.05</v>
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>3600000</v>
+        <v>947368</v>
       </c>
       <c r="K188" t="n">
-        <v>163964</v>
+        <v>104444</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9887,19 +9887,19 @@
         </is>
       </c>
       <c r="C189" s="89" t="n">
-        <v>359187</v>
+        <v>359188</v>
       </c>
       <c r="D189" s="89" t="n">
-        <v>791666</v>
+        <v>791667</v>
       </c>
       <c r="E189" s="79" t="n">
         <v>-0.5462894484210528</v>
       </c>
       <c r="F189" s="89" t="n">
-        <v>35180150</v>
+        <v>35180151</v>
       </c>
       <c r="G189" s="89" t="n">
-        <v>36518056</v>
+        <v>36518057</v>
       </c>
       <c r="H189" s="79" t="n">
         <v>-0.04</v>
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>3800000</v>
+        <v>1000000</v>
       </c>
       <c r="K189" t="n">
-        <v>172040</v>
+        <v>106802</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">
@@ -9933,7 +9933,7 @@
       </c>
       <c r="E190" s="79" t="n"/>
       <c r="F190" s="89" t="n">
-        <v>6210835</v>
+        <v>6210836</v>
       </c>
       <c r="G190" s="89" t="n">
         <v>6069577</v>
@@ -9948,7 +9948,7 @@
         <v>0</v>
       </c>
       <c r="K190" t="n">
-        <v>-5967</v>
+        <v>-19892</v>
       </c>
     </row>
     <row r="191" ht="14.25" customHeight="1" s="250">
@@ -9985,7 +9985,7 @@
         <v>0</v>
       </c>
       <c r="K191" t="n">
-        <v>-71</v>
+        <v>-238</v>
       </c>
     </row>
     <row r="192" ht="14.25" customHeight="1" s="250">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="E193" s="79" t="n"/>
       <c r="F193" s="89" t="n">
-        <v>6553840</v>
+        <v>6553841</v>
       </c>
       <c r="G193" s="89" t="n">
         <v>6381222</v>
@@ -10061,7 +10061,7 @@
         <v>0</v>
       </c>
       <c r="K193" t="n">
-        <v>-3613</v>
+        <v>-12045</v>
       </c>
     </row>
     <row r="194" ht="14.25" customHeight="1" s="250"/>
@@ -10221,10 +10221,10 @@
         <v>0.159622112638379</v>
       </c>
       <c r="H2" t="n">
-        <v>23</v>
+        <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -10252,10 +10252,10 @@
         <v>0.13006246214979</v>
       </c>
       <c r="H3" t="n">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="I3" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="250">
@@ -10283,10 +10283,10 @@
         <v>0.12785218855059</v>
       </c>
       <c r="H4" t="n">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="I4" t="n">
-        <v>22</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="250">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="G5" s="258" t="n"/>
       <c r="I5" t="n">
-        <v>29</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="250">
@@ -10338,10 +10338,10 @@
         <v>0.119182965859955</v>
       </c>
       <c r="H6" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="I6" t="n">
-        <v>23</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="250" thickBot="1">
@@ -10369,10 +10369,10 @@
         <v>0.106909295617267</v>
       </c>
       <c r="H7" t="n">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="I7" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="158">
@@ -10400,10 +10400,10 @@
         <v>0.127185196510197</v>
       </c>
       <c r="H8" t="n">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="I8" t="n">
-        <v>24</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="250">
@@ -10431,10 +10431,10 @@
         <v>0.130798384540069</v>
       </c>
       <c r="H9" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="I9" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="250">
@@ -10462,10 +10462,10 @@
         <v>0.197218920214015</v>
       </c>
       <c r="H10" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="I10" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="250">
@@ -10493,10 +10493,10 @@
         <v>0.156143076621019</v>
       </c>
       <c r="H11" t="n">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="I11" t="n">
-        <v>15</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="250">
@@ -10524,10 +10524,10 @@
         <v>0.125550416455854</v>
       </c>
       <c r="H12" t="n">
-        <v>229</v>
+        <v>764</v>
       </c>
       <c r="I12" t="n">
-        <v>207</v>
+        <v>692</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="250">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="G13" s="258" t="n"/>
       <c r="I13" t="n">
-        <v>31</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="250">
@@ -10579,10 +10579,10 @@
         <v>0.0806766817717267</v>
       </c>
       <c r="H14" t="n">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="I14" t="n">
-        <v>27</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="250">
@@ -10610,10 +10610,10 @@
         <v>0.0777021675916213</v>
       </c>
       <c r="H15" t="n">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="I15" t="n">
-        <v>32</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="250">
@@ -10637,7 +10637,7 @@
       </c>
       <c r="G16" s="260" t="n"/>
       <c r="I16" t="n">
-        <v>25</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="250">
@@ -10665,10 +10665,10 @@
         <v>0.095303991140541</v>
       </c>
       <c r="H17" t="n">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="I17" t="n">
-        <v>26</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="250">
@@ -10696,10 +10696,10 @@
         <v>0.0776551038922926</v>
       </c>
       <c r="H18" t="n">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="I18" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="250">
@@ -10727,10 +10727,10 @@
         <v>0.162114464314885</v>
       </c>
       <c r="H19" t="n">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="I19" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="250">
@@ -10754,7 +10754,7 @@
       </c>
       <c r="G20" s="208" t="n"/>
       <c r="I20" t="n">
-        <v>32</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="250">
@@ -10782,10 +10782,10 @@
         <v>0.08919891687813671</v>
       </c>
       <c r="H21" t="n">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="I21" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="250">
@@ -10813,10 +10813,10 @@
         <v>0.08301513631583469</v>
       </c>
       <c r="H22" t="n">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="I22" t="n">
-        <v>22</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="250">
@@ -10844,10 +10844,10 @@
         <v>0.06665486782805979</v>
       </c>
       <c r="H23" t="n">
-        <v>286</v>
+        <v>954</v>
       </c>
       <c r="I23" t="n">
-        <v>271</v>
+        <v>905</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="250">
@@ -10875,10 +10875,10 @@
         <v>0.07487484353666519</v>
       </c>
       <c r="H24" t="n">
-        <v>551</v>
+        <v>1836</v>
       </c>
       <c r="I24" t="n">
-        <v>508</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="250">

</xml_diff>

<commit_message>
feat: integrate Google Gmail API stock sync, n8n webhook, automatic trashing, and Telegram notifications
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2961,10 +2961,10 @@
         <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>10227</v>
+        <v>9375</v>
       </c>
       <c r="K10" t="n">
-        <v>36</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K11" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>5455</v>
+        <v>5000</v>
       </c>
       <c r="K12" t="n">
-        <v>212</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3230,10 +3230,10 @@
         <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>29545</v>
+        <v>27083</v>
       </c>
       <c r="K17" t="n">
-        <v>401</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3380,10 +3380,10 @@
         <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>10227</v>
+        <v>9375</v>
       </c>
       <c r="K21" t="n">
-        <v>41</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>7955</v>
+        <v>7292</v>
       </c>
       <c r="K22" t="n">
-        <v>61</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3458,10 +3458,10 @@
         <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K23" t="n">
-        <v>-17</v>
+        <v>-28</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>28409</v>
+        <v>26042</v>
       </c>
       <c r="K25" t="n">
-        <v>76</v>
+        <v>-42</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3575,10 +3575,10 @@
         <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>11364</v>
+        <v>10417</v>
       </c>
       <c r="K26" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3614,10 +3614,10 @@
         <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K27" t="n">
-        <v>-31</v>
+        <v>-40</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3653,10 +3653,10 @@
         <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K28" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3848,10 +3848,10 @@
         <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>31818</v>
+        <v>29167</v>
       </c>
       <c r="K33" t="n">
-        <v>-1126</v>
+        <v>-1258</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>12500</v>
+        <v>11458</v>
       </c>
       <c r="K37" t="n">
-        <v>625</v>
+        <v>573</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>6818</v>
+        <v>6250</v>
       </c>
       <c r="K38" t="n">
-        <v>341</v>
+        <v>312</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K39" t="n">
-        <v>170</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>29545</v>
+        <v>27083</v>
       </c>
       <c r="K41" t="n">
-        <v>1477</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>7955</v>
+        <v>7292</v>
       </c>
       <c r="K42" t="n">
-        <v>240</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K43" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>2045</v>
+        <v>1875</v>
       </c>
       <c r="K44" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>9091</v>
+        <v>8333</v>
       </c>
       <c r="K45" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K46" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K47" t="n">
-        <v>5</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>32955</v>
+        <v>30208</v>
       </c>
       <c r="K49" t="n">
-        <v>432</v>
+        <v>294</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>13636</v>
+        <v>12500</v>
       </c>
       <c r="K50" t="n">
-        <v>201</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>2955</v>
+        <v>2708</v>
       </c>
       <c r="K51" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K52" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>13636</v>
+        <v>12500</v>
       </c>
       <c r="K53" t="n">
-        <v>255</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>10227</v>
+        <v>9375</v>
       </c>
       <c r="K54" t="n">
-        <v>233</v>
+        <v>191</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K55" t="n">
-        <v>70</v>
+        <v>46</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>59091</v>
+        <v>54167</v>
       </c>
       <c r="K57" t="n">
-        <v>563</v>
+        <v>317</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>10227</v>
+        <v>9375</v>
       </c>
       <c r="K58" t="n">
-        <v>330</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4856,10 +4856,10 @@
         <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K59" t="n">
-        <v>71</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>3636</v>
+        <v>3333</v>
       </c>
       <c r="K60" t="n">
-        <v>128</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4934,10 +4934,10 @@
         <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>9091</v>
+        <v>8333</v>
       </c>
       <c r="K61" t="n">
-        <v>116</v>
+        <v>78</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4973,10 +4973,10 @@
         <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K62" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K63" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>38636</v>
+        <v>35417</v>
       </c>
       <c r="K65" t="n">
-        <v>635</v>
+        <v>474</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K66" t="n">
-        <v>284</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K67" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K68" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>7955</v>
+        <v>7292</v>
       </c>
       <c r="K69" t="n">
-        <v>398</v>
+        <v>365</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K70" t="n">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K71" t="n">
-        <v>284</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>31818</v>
+        <v>29167</v>
       </c>
       <c r="K73" t="n">
-        <v>1591</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>13636</v>
+        <v>12500</v>
       </c>
       <c r="K74" t="n">
-        <v>397</v>
+        <v>341</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>2955</v>
+        <v>2708</v>
       </c>
       <c r="K75" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>6818</v>
+        <v>6250</v>
       </c>
       <c r="K76" t="n">
-        <v>242</v>
+        <v>213</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5712,10 +5712,10 @@
         <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>34091</v>
+        <v>31250</v>
       </c>
       <c r="K81" t="n">
-        <v>-169</v>
+        <v>-311</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>9773</v>
+        <v>8958</v>
       </c>
       <c r="K85" t="n">
-        <v>489</v>
+        <v>448</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>5227</v>
+        <v>4792</v>
       </c>
       <c r="K86" t="n">
-        <v>261</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K87" t="n">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>27955</v>
+        <v>25625</v>
       </c>
       <c r="K89" t="n">
-        <v>1398</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>15909</v>
+        <v>14583</v>
       </c>
       <c r="K90" t="n">
-        <v>340</v>
+        <v>274</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K91" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>2727</v>
+        <v>2500</v>
       </c>
       <c r="K92" t="n">
-        <v>-53</v>
+        <v>-65</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6324,10 +6324,10 @@
         <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>34091</v>
+        <v>31250</v>
       </c>
       <c r="K97" t="n">
-        <v>435</v>
+        <v>293</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>18182</v>
+        <v>16667</v>
       </c>
       <c r="K101" t="n">
-        <v>372</v>
+        <v>297</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6513,10 +6513,10 @@
         <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>9091</v>
+        <v>8333</v>
       </c>
       <c r="K102" t="n">
-        <v>189</v>
+        <v>151</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6552,10 +6552,10 @@
         <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>5909</v>
+        <v>5417</v>
       </c>
       <c r="K103" t="n">
-        <v>-110</v>
+        <v>-135</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6630,10 +6630,10 @@
         <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>40909</v>
+        <v>37500</v>
       </c>
       <c r="K105" t="n">
-        <v>361</v>
+        <v>190</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>18182</v>
+        <v>16667</v>
       </c>
       <c r="K109" t="n">
-        <v>349</v>
+        <v>274</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6819,10 +6819,10 @@
         <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>10227</v>
+        <v>9375</v>
       </c>
       <c r="K110" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6858,10 +6858,10 @@
         <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K111" t="n">
-        <v>-51</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6936,10 +6936,10 @@
         <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>40909</v>
+        <v>37500</v>
       </c>
       <c r="K113" t="n">
-        <v>-2</v>
+        <v>-172</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6975,10 +6975,10 @@
         <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>14773</v>
+        <v>13542</v>
       </c>
       <c r="K114" t="n">
-        <v>-94</v>
+        <v>-156</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7014,10 +7014,10 @@
         <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>4545</v>
+        <v>4167</v>
       </c>
       <c r="K115" t="n">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K116" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7248,10 +7248,10 @@
         <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>34091</v>
+        <v>31250</v>
       </c>
       <c r="K121" t="n">
-        <v>-152</v>
+        <v>-294</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>15455</v>
+        <v>14167</v>
       </c>
       <c r="K122" t="n">
-        <v>204</v>
+        <v>140</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K123" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K124" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>17045</v>
+        <v>15625</v>
       </c>
       <c r="K125" t="n">
-        <v>214</v>
+        <v>143</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>7273</v>
+        <v>6667</v>
       </c>
       <c r="K126" t="n">
-        <v>-187</v>
+        <v>-217</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K127" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>63636</v>
+        <v>58333</v>
       </c>
       <c r="K129" t="n">
-        <v>458</v>
+        <v>193</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>4545</v>
+        <v>4167</v>
       </c>
       <c r="K130" t="n">
-        <v>-82</v>
+        <v>-101</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K131" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K132" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>5682</v>
+        <v>5208</v>
       </c>
       <c r="K133" t="n">
-        <v>1</v>
+        <v>-23</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K134" t="n">
-        <v>-45</v>
+        <v>-59</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K135" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>31818</v>
+        <v>29167</v>
       </c>
       <c r="K137" t="n">
-        <v>-56</v>
+        <v>-188</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>4545</v>
+        <v>4167</v>
       </c>
       <c r="K138" t="n">
-        <v>-81</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K139" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K140" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>6818</v>
+        <v>6250</v>
       </c>
       <c r="K141" t="n">
-        <v>3</v>
+        <v>-25</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K142" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K143" t="n">
-        <v>83</v>
+        <v>69</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>34091</v>
+        <v>31250</v>
       </c>
       <c r="K145" t="n">
-        <v>357</v>
+        <v>215</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>7955</v>
+        <v>7292</v>
       </c>
       <c r="K146" t="n">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K147" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>2841</v>
+        <v>2604</v>
       </c>
       <c r="K148" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>9091</v>
+        <v>8333</v>
       </c>
       <c r="K149" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>4545</v>
+        <v>4167</v>
       </c>
       <c r="K150" t="n">
-        <v>-5</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>3409</v>
+        <v>3125</v>
       </c>
       <c r="K151" t="n">
-        <v>6</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>34091</v>
+        <v>31250</v>
       </c>
       <c r="K153" t="n">
-        <v>40</v>
+        <v>-102</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>6818</v>
+        <v>6250</v>
       </c>
       <c r="K154" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8588,10 +8588,10 @@
         <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K155" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8627,10 +8627,10 @@
         <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>2273</v>
+        <v>2083</v>
       </c>
       <c r="K156" t="n">
-        <v>3</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>27273</v>
+        <v>25000</v>
       </c>
       <c r="K161" t="n">
-        <v>-476</v>
+        <v>-590</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>14773</v>
+        <v>13542</v>
       </c>
       <c r="K165" t="n">
-        <v>739</v>
+        <v>677</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>8636</v>
+        <v>7917</v>
       </c>
       <c r="K166" t="n">
-        <v>432</v>
+        <v>396</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>6364</v>
+        <v>5833</v>
       </c>
       <c r="K167" t="n">
-        <v>318</v>
+        <v>292</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>37955</v>
+        <v>34792</v>
       </c>
       <c r="K169" t="n">
-        <v>1898</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9167,10 +9167,10 @@
         <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>169318</v>
+        <v>155208</v>
       </c>
       <c r="K170" t="n">
-        <v>7463</v>
+        <v>6758</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9206,10 +9206,10 @@
         <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>40909</v>
+        <v>37500</v>
       </c>
       <c r="K171" t="n">
-        <v>406</v>
+        <v>236</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9245,10 +9245,10 @@
         <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>30682</v>
+        <v>28125</v>
       </c>
       <c r="K172" t="n">
-        <v>1403</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>420455</v>
+        <v>385417</v>
       </c>
       <c r="K173" t="n">
-        <v>19284</v>
+        <v>17532</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9323,10 +9323,10 @@
         <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>21591</v>
+        <v>19792</v>
       </c>
       <c r="K174" t="n">
-        <v>291</v>
+        <v>201</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>21591</v>
+        <v>19792</v>
       </c>
       <c r="K175" t="n">
-        <v>800</v>
+        <v>710</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>968182</v>
+        <v>887500</v>
       </c>
       <c r="K177" t="n">
-        <v>35889</v>
+        <v>31855</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9479,10 +9479,10 @@
         <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>72727</v>
+        <v>66667</v>
       </c>
       <c r="K178" t="n">
-        <v>1539</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9518,10 +9518,10 @@
         <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>18182</v>
+        <v>16667</v>
       </c>
       <c r="K179" t="n">
-        <v>362</v>
+        <v>286</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9557,10 +9557,10 @@
         <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>26364</v>
+        <v>24167</v>
       </c>
       <c r="K180" t="n">
-        <v>885</v>
+        <v>775</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9596,10 +9596,10 @@
         <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>72273</v>
+        <v>66250</v>
       </c>
       <c r="K181" t="n">
-        <v>991</v>
+        <v>690</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>41364</v>
+        <v>37917</v>
       </c>
       <c r="K182" t="n">
-        <v>521</v>
+        <v>349</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>24773</v>
+        <v>22708</v>
       </c>
       <c r="K183" t="n">
-        <v>344</v>
+        <v>240</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>343864</v>
+        <v>315208</v>
       </c>
       <c r="K185" t="n">
-        <v>5279</v>
+        <v>3846</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>1690909</v>
+        <v>1550000</v>
       </c>
       <c r="K187" t="n">
-        <v>44032</v>
+        <v>36986</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>818182</v>
+        <v>750000</v>
       </c>
       <c r="K188" t="n">
-        <v>24874</v>
+        <v>21465</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>863636</v>
+        <v>791667</v>
       </c>
       <c r="K189" t="n">
-        <v>25222</v>
+        <v>21624</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">

</xml_diff>

<commit_message>
fix: double-counting, remove duplicate chart, add suivi terrain filters & totals, reload latest date, override html2canvas 1.4.1 for CSS variable compatibility, add safety timeouts
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2664,7 +2664,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>-592</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>-1520</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="250">
@@ -2775,7 +2775,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>-208</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="250">
@@ -2812,7 +2812,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>-342</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2925,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>-8036</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="250">
@@ -2961,10 +2961,10 @@
         <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>9375</v>
+        <v>25000</v>
       </c>
       <c r="K10" t="n">
-        <v>-7</v>
+        <v>774</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K11" t="n">
-        <v>63</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>5000</v>
+        <v>13333</v>
       </c>
       <c r="K12" t="n">
-        <v>189</v>
+        <v>606</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3230,10 +3230,10 @@
         <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>27083</v>
+        <v>72222</v>
       </c>
       <c r="K17" t="n">
-        <v>278</v>
+        <v>2535</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3380,10 +3380,10 @@
         <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>9375</v>
+        <v>25000</v>
       </c>
       <c r="K21" t="n">
-        <v>-2</v>
+        <v>779</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>7292</v>
+        <v>19444</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>635</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3458,10 +3458,10 @@
         <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K23" t="n">
-        <v>-28</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>26042</v>
+        <v>69444</v>
       </c>
       <c r="K25" t="n">
-        <v>-42</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3575,10 +3575,10 @@
         <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>10417</v>
+        <v>27778</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>872</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3614,10 +3614,10 @@
         <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K27" t="n">
-        <v>-40</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3653,10 +3653,10 @@
         <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K28" t="n">
-        <v>25</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3695,7 +3695,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>-629</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="14.25" customHeight="1" s="250">
@@ -3734,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>-318</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="14.25" customHeight="1" s="250">
@@ -3773,7 +3773,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>-229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="250">
@@ -3848,10 +3848,10 @@
         <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>29167</v>
+        <v>77778</v>
       </c>
       <c r="K33" t="n">
-        <v>-1258</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>11458</v>
+        <v>30556</v>
       </c>
       <c r="K37" t="n">
-        <v>573</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>6250</v>
+        <v>16667</v>
       </c>
       <c r="K38" t="n">
-        <v>312</v>
+        <v>833</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K39" t="n">
-        <v>156</v>
+        <v>417</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>27083</v>
+        <v>72222</v>
       </c>
       <c r="K41" t="n">
-        <v>1354</v>
+        <v>3611</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>7292</v>
+        <v>19444</v>
       </c>
       <c r="K42" t="n">
-        <v>206</v>
+        <v>814</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K43" t="n">
-        <v>40</v>
+        <v>213</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1875</v>
+        <v>5000</v>
       </c>
       <c r="K44" t="n">
-        <v>88</v>
+        <v>244</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>8333</v>
+        <v>22222</v>
       </c>
       <c r="K45" t="n">
-        <v>86</v>
+        <v>780</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K46" t="n">
-        <v>10</v>
+        <v>444</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K47" t="n">
-        <v>-5</v>
+        <v>169</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>30208</v>
+        <v>80556</v>
       </c>
       <c r="K49" t="n">
-        <v>294</v>
+        <v>2812</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>12500</v>
+        <v>33333</v>
       </c>
       <c r="K50" t="n">
-        <v>144</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>2708</v>
+        <v>7222</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>229</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K52" t="n">
-        <v>43</v>
+        <v>303</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>12500</v>
+        <v>33333</v>
       </c>
       <c r="K53" t="n">
-        <v>198</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>9375</v>
+        <v>25000</v>
       </c>
       <c r="K54" t="n">
-        <v>191</v>
+        <v>972</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K55" t="n">
-        <v>46</v>
+        <v>480</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>54167</v>
+        <v>144444</v>
       </c>
       <c r="K57" t="n">
-        <v>317</v>
+        <v>4830</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>9375</v>
+        <v>25000</v>
       </c>
       <c r="K58" t="n">
-        <v>288</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4856,10 +4856,10 @@
         <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K59" t="n">
-        <v>60</v>
+        <v>268</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>3333</v>
+        <v>8889</v>
       </c>
       <c r="K60" t="n">
-        <v>113</v>
+        <v>391</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4934,10 +4934,10 @@
         <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>8333</v>
+        <v>22222</v>
       </c>
       <c r="K61" t="n">
-        <v>78</v>
+        <v>772</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4973,10 +4973,10 @@
         <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K62" t="n">
-        <v>5</v>
+        <v>213</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K63" t="n">
-        <v>37</v>
+        <v>211</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>35417</v>
+        <v>94444</v>
       </c>
       <c r="K65" t="n">
-        <v>474</v>
+        <v>3426</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K66" t="n">
-        <v>260</v>
+        <v>694</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K67" t="n">
-        <v>104</v>
+        <v>278</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K68" t="n">
-        <v>104</v>
+        <v>278</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>7292</v>
+        <v>19444</v>
       </c>
       <c r="K69" t="n">
-        <v>365</v>
+        <v>972</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K70" t="n">
-        <v>125</v>
+        <v>333</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K71" t="n">
-        <v>260</v>
+        <v>694</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>29167</v>
+        <v>77778</v>
       </c>
       <c r="K73" t="n">
-        <v>1458</v>
+        <v>3889</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>12500</v>
+        <v>33333</v>
       </c>
       <c r="K74" t="n">
-        <v>341</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>2708</v>
+        <v>7222</v>
       </c>
       <c r="K75" t="n">
-        <v>57</v>
+        <v>282</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>6250</v>
+        <v>16667</v>
       </c>
       <c r="K76" t="n">
-        <v>213</v>
+        <v>734</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5561,7 +5561,7 @@
         <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>-426</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" ht="14.25" customHeight="1" s="250">
@@ -5598,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>-243</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" ht="14.25" customHeight="1" s="250">
@@ -5637,7 +5637,7 @@
         <v>0</v>
       </c>
       <c r="K79" t="n">
-        <v>-123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" ht="14.25" customHeight="1" s="250">
@@ -5712,10 +5712,10 @@
         <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>31250</v>
+        <v>83333</v>
       </c>
       <c r="K81" t="n">
-        <v>-311</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>8958</v>
+        <v>23889</v>
       </c>
       <c r="K85" t="n">
-        <v>448</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>4792</v>
+        <v>12778</v>
       </c>
       <c r="K86" t="n">
-        <v>240</v>
+        <v>639</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K87" t="n">
-        <v>125</v>
+        <v>333</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>25625</v>
+        <v>68333</v>
       </c>
       <c r="K89" t="n">
-        <v>1281</v>
+        <v>3417</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>14583</v>
+        <v>38889</v>
       </c>
       <c r="K90" t="n">
-        <v>274</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>2500</v>
+        <v>6667</v>
       </c>
       <c r="K92" t="n">
-        <v>-65</v>
+        <v>144</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6324,10 +6324,10 @@
         <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>31250</v>
+        <v>83333</v>
       </c>
       <c r="K97" t="n">
-        <v>293</v>
+        <v>2897</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>16667</v>
+        <v>44444</v>
       </c>
       <c r="K101" t="n">
-        <v>297</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6513,10 +6513,10 @@
         <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>8333</v>
+        <v>22222</v>
       </c>
       <c r="K102" t="n">
-        <v>151</v>
+        <v>846</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6552,10 +6552,10 @@
         <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>5417</v>
+        <v>14444</v>
       </c>
       <c r="K103" t="n">
-        <v>-135</v>
+        <v>316</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6630,10 +6630,10 @@
         <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>37500</v>
+        <v>100000</v>
       </c>
       <c r="K105" t="n">
-        <v>190</v>
+        <v>3315</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>16667</v>
+        <v>44444</v>
       </c>
       <c r="K109" t="n">
-        <v>274</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6819,10 +6819,10 @@
         <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>9375</v>
+        <v>25000</v>
       </c>
       <c r="K110" t="n">
-        <v>40</v>
+        <v>821</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6858,10 +6858,10 @@
         <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K111" t="n">
-        <v>-75</v>
+        <v>359</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6936,10 +6936,10 @@
         <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>37500</v>
+        <v>100000</v>
       </c>
       <c r="K113" t="n">
-        <v>-172</v>
+        <v>2953</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6975,10 +6975,10 @@
         <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>13542</v>
+        <v>36111</v>
       </c>
       <c r="K114" t="n">
-        <v>-156</v>
+        <v>973</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7014,10 +7014,10 @@
         <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>4167</v>
+        <v>11111</v>
       </c>
       <c r="K115" t="n">
-        <v>73</v>
+        <v>420</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K116" t="n">
-        <v>29</v>
+        <v>463</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7248,10 +7248,10 @@
         <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>31250</v>
+        <v>83333</v>
       </c>
       <c r="K121" t="n">
-        <v>-294</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>14167</v>
+        <v>37778</v>
       </c>
       <c r="K122" t="n">
-        <v>140</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K123" t="n">
-        <v>96</v>
+        <v>357</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K124" t="n">
-        <v>51</v>
+        <v>224</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>15625</v>
+        <v>41667</v>
       </c>
       <c r="K125" t="n">
-        <v>143</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>6667</v>
+        <v>17778</v>
       </c>
       <c r="K126" t="n">
-        <v>-217</v>
+        <v>338</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K127" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>58333</v>
+        <v>155556</v>
       </c>
       <c r="K129" t="n">
-        <v>193</v>
+        <v>5054</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>4167</v>
+        <v>11111</v>
       </c>
       <c r="K130" t="n">
-        <v>-101</v>
+        <v>247</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K131" t="n">
-        <v>52</v>
+        <v>225</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K132" t="n">
-        <v>50</v>
+        <v>224</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>5208</v>
+        <v>13889</v>
       </c>
       <c r="K133" t="n">
-        <v>-23</v>
+        <v>411</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K134" t="n">
-        <v>-59</v>
+        <v>201</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K135" t="n">
-        <v>3</v>
+        <v>176</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>29167</v>
+        <v>77778</v>
       </c>
       <c r="K137" t="n">
-        <v>-188</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>4167</v>
+        <v>11111</v>
       </c>
       <c r="K138" t="n">
-        <v>-100</v>
+        <v>248</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K139" t="n">
-        <v>42</v>
+        <v>215</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K140" t="n">
-        <v>92</v>
+        <v>266</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>6250</v>
+        <v>16667</v>
       </c>
       <c r="K141" t="n">
-        <v>-25</v>
+        <v>496</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K142" t="n">
-        <v>21</v>
+        <v>281</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K143" t="n">
-        <v>69</v>
+        <v>329</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>31250</v>
+        <v>83333</v>
       </c>
       <c r="K145" t="n">
-        <v>215</v>
+        <v>2820</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>7292</v>
+        <v>19444</v>
       </c>
       <c r="K146" t="n">
-        <v>49</v>
+        <v>657</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K147" t="n">
-        <v>61</v>
+        <v>234</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>2604</v>
+        <v>6944</v>
       </c>
       <c r="K148" t="n">
-        <v>78</v>
+        <v>295</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>8333</v>
+        <v>22222</v>
       </c>
       <c r="K149" t="n">
-        <v>17</v>
+        <v>712</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>4167</v>
+        <v>11111</v>
       </c>
       <c r="K150" t="n">
-        <v>-24</v>
+        <v>323</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>3125</v>
+        <v>8333</v>
       </c>
       <c r="K151" t="n">
-        <v>-9</v>
+        <v>252</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>31250</v>
+        <v>83333</v>
       </c>
       <c r="K153" t="n">
-        <v>-102</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>6250</v>
+        <v>16667</v>
       </c>
       <c r="K154" t="n">
-        <v>13</v>
+        <v>534</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8588,10 +8588,10 @@
         <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K155" t="n">
-        <v>5</v>
+        <v>179</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8627,10 +8627,10 @@
         <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>2083</v>
+        <v>5556</v>
       </c>
       <c r="K156" t="n">
-        <v>-6</v>
+        <v>167</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8669,7 +8669,7 @@
         <v>0</v>
       </c>
       <c r="K157" t="n">
-        <v>-348</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" ht="14.25" customHeight="1" s="250">
@@ -8708,7 +8708,7 @@
         <v>0</v>
       </c>
       <c r="K158" t="n">
-        <v>-171</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159" ht="14.25" customHeight="1" s="250">
@@ -8747,7 +8747,7 @@
         <v>0</v>
       </c>
       <c r="K159" t="n">
-        <v>-124</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" ht="14.25" customHeight="1" s="250">
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>25000</v>
+        <v>66667</v>
       </c>
       <c r="K161" t="n">
-        <v>-590</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>13542</v>
+        <v>36111</v>
       </c>
       <c r="K165" t="n">
-        <v>677</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>7917</v>
+        <v>21111</v>
       </c>
       <c r="K166" t="n">
-        <v>396</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>5833</v>
+        <v>15556</v>
       </c>
       <c r="K167" t="n">
-        <v>292</v>
+        <v>778</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>34792</v>
+        <v>92778</v>
       </c>
       <c r="K169" t="n">
-        <v>1740</v>
+        <v>4639</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9167,10 +9167,10 @@
         <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>155208</v>
+        <v>413889</v>
       </c>
       <c r="K170" t="n">
-        <v>6758</v>
+        <v>19692</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9206,10 +9206,10 @@
         <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>37500</v>
+        <v>100000</v>
       </c>
       <c r="K171" t="n">
-        <v>236</v>
+        <v>3361</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9245,10 +9245,10 @@
         <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>28125</v>
+        <v>75000</v>
       </c>
       <c r="K172" t="n">
-        <v>1276</v>
+        <v>3619</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>385417</v>
+        <v>1027778</v>
       </c>
       <c r="K173" t="n">
-        <v>17532</v>
+        <v>49650</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9323,10 +9323,10 @@
         <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>19792</v>
+        <v>52778</v>
       </c>
       <c r="K174" t="n">
-        <v>201</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>19792</v>
+        <v>52778</v>
       </c>
       <c r="K175" t="n">
-        <v>710</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>887500</v>
+        <v>2366667</v>
       </c>
       <c r="K177" t="n">
-        <v>31855</v>
+        <v>105814</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9479,10 +9479,10 @@
         <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>66667</v>
+        <v>177778</v>
       </c>
       <c r="K178" t="n">
-        <v>1236</v>
+        <v>6792</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9518,10 +9518,10 @@
         <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>16667</v>
+        <v>44444</v>
       </c>
       <c r="K179" t="n">
-        <v>286</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9557,10 +9557,10 @@
         <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>24167</v>
+        <v>64444</v>
       </c>
       <c r="K180" t="n">
-        <v>775</v>
+        <v>2789</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9596,10 +9596,10 @@
         <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>66250</v>
+        <v>176667</v>
       </c>
       <c r="K181" t="n">
-        <v>690</v>
+        <v>6211</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>37917</v>
+        <v>101111</v>
       </c>
       <c r="K182" t="n">
-        <v>349</v>
+        <v>3508</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>22708</v>
+        <v>60556</v>
       </c>
       <c r="K183" t="n">
-        <v>240</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>315208</v>
+        <v>840556</v>
       </c>
       <c r="K185" t="n">
-        <v>3846</v>
+        <v>30113</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>1550000</v>
+        <v>4133333</v>
       </c>
       <c r="K187" t="n">
-        <v>36986</v>
+        <v>166153</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>750000</v>
+        <v>2000000</v>
       </c>
       <c r="K188" t="n">
-        <v>21465</v>
+        <v>83965</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>791667</v>
+        <v>2111111</v>
       </c>
       <c r="K189" t="n">
-        <v>21624</v>
+        <v>87596</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">
@@ -9948,7 +9948,7 @@
         <v>0</v>
       </c>
       <c r="K190" t="n">
-        <v>-5968</v>
+        <v>0</v>
       </c>
     </row>
     <row r="191" ht="14.25" customHeight="1" s="250">
@@ -9985,7 +9985,7 @@
         <v>0</v>
       </c>
       <c r="K191" t="n">
-        <v>-71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="192" ht="14.25" customHeight="1" s="250">
@@ -10061,7 +10061,7 @@
         <v>0</v>
       </c>
       <c r="K193" t="n">
-        <v>-3614</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" ht="14.25" customHeight="1" s="250"/>
@@ -10502,7 +10502,7 @@
     <row r="12" ht="16.5" customHeight="1" s="250">
       <c r="A12" s="210" t="inlineStr">
         <is>
-          <t>BOUTMEZGUINE EL MOSTAFA</t>
+          <t>VIDE</t>
         </is>
       </c>
       <c r="B12" s="210" t="n">
@@ -10822,7 +10822,7 @@
     <row r="23" ht="16.5" customHeight="1" s="250">
       <c r="A23" s="210" t="inlineStr">
         <is>
-          <t>CHAKIB ELFIL</t>
+          <t>VIDE</t>
         </is>
       </c>
       <c r="B23" s="210" t="n">

</xml_diff>

<commit_message>
Update CDZ targets, team sellers count, Histo 2025/2026 columns and table layouts to match Excel model
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2961,10 +2961,10 @@
         <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>25000</v>
+        <v>9375</v>
       </c>
       <c r="K10" t="n">
-        <v>774</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K11" t="n">
-        <v>271</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>13333</v>
+        <v>5000</v>
       </c>
       <c r="K12" t="n">
-        <v>606</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3230,10 +3230,10 @@
         <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>72222</v>
+        <v>27083</v>
       </c>
       <c r="K17" t="n">
-        <v>2535</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3380,10 +3380,10 @@
         <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>25000</v>
+        <v>9375</v>
       </c>
       <c r="K21" t="n">
-        <v>779</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>19444</v>
+        <v>7292</v>
       </c>
       <c r="K22" t="n">
-        <v>635</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3458,10 +3458,10 @@
         <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K23" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>69444</v>
+        <v>26042</v>
       </c>
       <c r="K25" t="n">
-        <v>2128</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3575,10 +3575,10 @@
         <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>27778</v>
+        <v>10417</v>
       </c>
       <c r="K26" t="n">
-        <v>872</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3614,10 +3614,10 @@
         <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K27" t="n">
-        <v>134</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3653,10 +3653,10 @@
         <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K28" t="n">
-        <v>233</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3848,10 +3848,10 @@
         <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>77778</v>
+        <v>29167</v>
       </c>
       <c r="K33" t="n">
-        <v>1172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>30556</v>
+        <v>11458</v>
       </c>
       <c r="K37" t="n">
-        <v>1528</v>
+        <v>573</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>16667</v>
+        <v>6250</v>
       </c>
       <c r="K38" t="n">
-        <v>833</v>
+        <v>312</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K39" t="n">
-        <v>417</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>72222</v>
+        <v>27083</v>
       </c>
       <c r="K41" t="n">
-        <v>3611</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>19444</v>
+        <v>7292</v>
       </c>
       <c r="K42" t="n">
-        <v>814</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K43" t="n">
-        <v>213</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>5000</v>
+        <v>1875</v>
       </c>
       <c r="K44" t="n">
-        <v>244</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>22222</v>
+        <v>8333</v>
       </c>
       <c r="K45" t="n">
-        <v>780</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K46" t="n">
-        <v>444</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K47" t="n">
-        <v>169</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>80556</v>
+        <v>30208</v>
       </c>
       <c r="K49" t="n">
-        <v>2812</v>
+        <v>294</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>33333</v>
+        <v>12500</v>
       </c>
       <c r="K50" t="n">
-        <v>1186</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>7222</v>
+        <v>2708</v>
       </c>
       <c r="K51" t="n">
-        <v>229</v>
+        <v>3</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K52" t="n">
-        <v>303</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>33333</v>
+        <v>12500</v>
       </c>
       <c r="K53" t="n">
-        <v>1240</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>25000</v>
+        <v>9375</v>
       </c>
       <c r="K54" t="n">
-        <v>972</v>
+        <v>191</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K55" t="n">
-        <v>480</v>
+        <v>46</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>144444</v>
+        <v>54167</v>
       </c>
       <c r="K57" t="n">
-        <v>4830</v>
+        <v>317</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>25000</v>
+        <v>9375</v>
       </c>
       <c r="K58" t="n">
-        <v>1069</v>
+        <v>288</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4856,10 +4856,10 @@
         <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K59" t="n">
-        <v>268</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>8889</v>
+        <v>3333</v>
       </c>
       <c r="K60" t="n">
-        <v>391</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4934,10 +4934,10 @@
         <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>22222</v>
+        <v>8333</v>
       </c>
       <c r="K61" t="n">
-        <v>772</v>
+        <v>78</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4973,10 +4973,10 @@
         <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K62" t="n">
-        <v>213</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K63" t="n">
-        <v>211</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>94444</v>
+        <v>35417</v>
       </c>
       <c r="K65" t="n">
-        <v>3426</v>
+        <v>474</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K66" t="n">
-        <v>694</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K67" t="n">
-        <v>278</v>
+        <v>104</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K68" t="n">
-        <v>278</v>
+        <v>104</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>19444</v>
+        <v>7292</v>
       </c>
       <c r="K69" t="n">
-        <v>972</v>
+        <v>365</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K70" t="n">
-        <v>333</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K71" t="n">
-        <v>694</v>
+        <v>260</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>77778</v>
+        <v>29167</v>
       </c>
       <c r="K73" t="n">
-        <v>3889</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>33333</v>
+        <v>12500</v>
       </c>
       <c r="K74" t="n">
-        <v>1382</v>
+        <v>341</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>7222</v>
+        <v>2708</v>
       </c>
       <c r="K75" t="n">
-        <v>282</v>
+        <v>57</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>16667</v>
+        <v>6250</v>
       </c>
       <c r="K76" t="n">
-        <v>734</v>
+        <v>213</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5712,10 +5712,10 @@
         <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>83333</v>
+        <v>31250</v>
       </c>
       <c r="K81" t="n">
-        <v>2293</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>23889</v>
+        <v>8958</v>
       </c>
       <c r="K85" t="n">
-        <v>1194</v>
+        <v>448</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>12778</v>
+        <v>4792</v>
       </c>
       <c r="K86" t="n">
-        <v>639</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K87" t="n">
-        <v>333</v>
+        <v>125</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>68333</v>
+        <v>25625</v>
       </c>
       <c r="K89" t="n">
-        <v>3417</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>38889</v>
+        <v>14583</v>
       </c>
       <c r="K90" t="n">
-        <v>1489</v>
+        <v>274</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K91" t="n">
-        <v>174</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>6667</v>
+        <v>2500</v>
       </c>
       <c r="K92" t="n">
-        <v>144</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6324,10 +6324,10 @@
         <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>83333</v>
+        <v>31250</v>
       </c>
       <c r="K97" t="n">
-        <v>2897</v>
+        <v>293</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>44444</v>
+        <v>16667</v>
       </c>
       <c r="K101" t="n">
-        <v>1686</v>
+        <v>297</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6513,10 +6513,10 @@
         <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>22222</v>
+        <v>8333</v>
       </c>
       <c r="K102" t="n">
-        <v>846</v>
+        <v>151</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6552,10 +6552,10 @@
         <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>14444</v>
+        <v>5417</v>
       </c>
       <c r="K103" t="n">
-        <v>316</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6630,10 +6630,10 @@
         <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>100000</v>
+        <v>37500</v>
       </c>
       <c r="K105" t="n">
-        <v>3315</v>
+        <v>190</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>44444</v>
+        <v>16667</v>
       </c>
       <c r="K109" t="n">
-        <v>1662</v>
+        <v>274</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6819,10 +6819,10 @@
         <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>25000</v>
+        <v>9375</v>
       </c>
       <c r="K110" t="n">
-        <v>821</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6858,10 +6858,10 @@
         <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K111" t="n">
-        <v>359</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6936,10 +6936,10 @@
         <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>100000</v>
+        <v>37500</v>
       </c>
       <c r="K113" t="n">
-        <v>2953</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6975,10 +6975,10 @@
         <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>36111</v>
+        <v>13542</v>
       </c>
       <c r="K114" t="n">
-        <v>973</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7014,10 +7014,10 @@
         <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>11111</v>
+        <v>4167</v>
       </c>
       <c r="K115" t="n">
-        <v>420</v>
+        <v>73</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K116" t="n">
-        <v>463</v>
+        <v>29</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7248,10 +7248,10 @@
         <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>83333</v>
+        <v>31250</v>
       </c>
       <c r="K121" t="n">
-        <v>2310</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>37778</v>
+        <v>14167</v>
       </c>
       <c r="K122" t="n">
-        <v>1320</v>
+        <v>140</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K123" t="n">
-        <v>357</v>
+        <v>96</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K124" t="n">
-        <v>224</v>
+        <v>51</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>41667</v>
+        <v>15625</v>
       </c>
       <c r="K125" t="n">
-        <v>1445</v>
+        <v>143</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>17778</v>
+        <v>6667</v>
       </c>
       <c r="K126" t="n">
-        <v>338</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K127" t="n">
-        <v>173</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>155556</v>
+        <v>58333</v>
       </c>
       <c r="K129" t="n">
-        <v>5054</v>
+        <v>193</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>11111</v>
+        <v>4167</v>
       </c>
       <c r="K130" t="n">
-        <v>247</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K131" t="n">
-        <v>225</v>
+        <v>52</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K132" t="n">
-        <v>224</v>
+        <v>50</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>13889</v>
+        <v>5208</v>
       </c>
       <c r="K133" t="n">
-        <v>411</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K134" t="n">
-        <v>201</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K135" t="n">
-        <v>176</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>77778</v>
+        <v>29167</v>
       </c>
       <c r="K137" t="n">
-        <v>2242</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>11111</v>
+        <v>4167</v>
       </c>
       <c r="K138" t="n">
-        <v>248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K139" t="n">
-        <v>215</v>
+        <v>42</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K140" t="n">
-        <v>266</v>
+        <v>92</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>16667</v>
+        <v>6250</v>
       </c>
       <c r="K141" t="n">
-        <v>496</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K142" t="n">
-        <v>281</v>
+        <v>21</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K143" t="n">
-        <v>329</v>
+        <v>69</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>83333</v>
+        <v>31250</v>
       </c>
       <c r="K145" t="n">
-        <v>2820</v>
+        <v>215</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>19444</v>
+        <v>7292</v>
       </c>
       <c r="K146" t="n">
-        <v>657</v>
+        <v>49</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K147" t="n">
-        <v>234</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>6944</v>
+        <v>2604</v>
       </c>
       <c r="K148" t="n">
-        <v>295</v>
+        <v>78</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>22222</v>
+        <v>8333</v>
       </c>
       <c r="K149" t="n">
-        <v>712</v>
+        <v>17</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>11111</v>
+        <v>4167</v>
       </c>
       <c r="K150" t="n">
-        <v>323</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>8333</v>
+        <v>3125</v>
       </c>
       <c r="K151" t="n">
-        <v>252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>83333</v>
+        <v>31250</v>
       </c>
       <c r="K153" t="n">
-        <v>2503</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>16667</v>
+        <v>6250</v>
       </c>
       <c r="K154" t="n">
-        <v>534</v>
+        <v>13</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8588,10 +8588,10 @@
         <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K155" t="n">
-        <v>179</v>
+        <v>5</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8627,10 +8627,10 @@
         <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>5556</v>
+        <v>2083</v>
       </c>
       <c r="K156" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>66667</v>
+        <v>25000</v>
       </c>
       <c r="K161" t="n">
-        <v>1493</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>36111</v>
+        <v>13542</v>
       </c>
       <c r="K165" t="n">
-        <v>1806</v>
+        <v>677</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>21111</v>
+        <v>7917</v>
       </c>
       <c r="K166" t="n">
-        <v>1056</v>
+        <v>396</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>15556</v>
+        <v>5833</v>
       </c>
       <c r="K167" t="n">
-        <v>778</v>
+        <v>292</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>92778</v>
+        <v>34792</v>
       </c>
       <c r="K169" t="n">
-        <v>4639</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9167,10 +9167,10 @@
         <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>413889</v>
+        <v>155208</v>
       </c>
       <c r="K170" t="n">
-        <v>19692</v>
+        <v>6758</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9206,10 +9206,10 @@
         <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>100000</v>
+        <v>37500</v>
       </c>
       <c r="K171" t="n">
-        <v>3361</v>
+        <v>236</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9245,10 +9245,10 @@
         <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>75000</v>
+        <v>28125</v>
       </c>
       <c r="K172" t="n">
-        <v>3619</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>1027778</v>
+        <v>385417</v>
       </c>
       <c r="K173" t="n">
-        <v>49650</v>
+        <v>17532</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9323,10 +9323,10 @@
         <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>52778</v>
+        <v>19792</v>
       </c>
       <c r="K174" t="n">
-        <v>1850</v>
+        <v>201</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>52778</v>
+        <v>19792</v>
       </c>
       <c r="K175" t="n">
-        <v>2359</v>
+        <v>710</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>2366667</v>
+        <v>887500</v>
       </c>
       <c r="K177" t="n">
-        <v>105814</v>
+        <v>31855</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9479,10 +9479,10 @@
         <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>177778</v>
+        <v>66667</v>
       </c>
       <c r="K178" t="n">
-        <v>6792</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9518,10 +9518,10 @@
         <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>44444</v>
+        <v>16667</v>
       </c>
       <c r="K179" t="n">
-        <v>1675</v>
+        <v>286</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9557,10 +9557,10 @@
         <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>64444</v>
+        <v>24167</v>
       </c>
       <c r="K180" t="n">
-        <v>2789</v>
+        <v>775</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9596,10 +9596,10 @@
         <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>176667</v>
+        <v>66250</v>
       </c>
       <c r="K181" t="n">
-        <v>6211</v>
+        <v>690</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>101111</v>
+        <v>37917</v>
       </c>
       <c r="K182" t="n">
-        <v>3508</v>
+        <v>349</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>60556</v>
+        <v>22708</v>
       </c>
       <c r="K183" t="n">
-        <v>2133</v>
+        <v>240</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>840556</v>
+        <v>315208</v>
       </c>
       <c r="K185" t="n">
-        <v>30113</v>
+        <v>3846</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>4133333</v>
+        <v>1550000</v>
       </c>
       <c r="K187" t="n">
-        <v>166153</v>
+        <v>36986</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>2000000</v>
+        <v>750000</v>
       </c>
       <c r="K188" t="n">
-        <v>83965</v>
+        <v>21465</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>2111111</v>
+        <v>791667</v>
       </c>
       <c r="K189" t="n">
-        <v>87596</v>
+        <v>21624</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">

</xml_diff>

<commit_message>
Deploy: Login authentication modal, security headers, vendor active days count, interactive anomaly exclusions
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2961,10 +2961,10 @@
         <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>9375</v>
+        <v>37500</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K11" t="n">
-        <v>63</v>
+        <v>438</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="K12" t="n">
-        <v>189</v>
+        <v>939</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3230,10 +3230,10 @@
         <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>27083</v>
+        <v>108333</v>
       </c>
       <c r="K17" t="n">
-        <v>278</v>
+        <v>4341</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3380,10 +3380,10 @@
         <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>9375</v>
+        <v>37500</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>7292</v>
+        <v>29167</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3458,10 +3458,10 @@
         <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>347</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>26042</v>
+        <v>104167</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>3864</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3575,10 +3575,10 @@
         <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>10417</v>
+        <v>41667</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3614,10 +3614,10 @@
         <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>272</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3653,10 +3653,10 @@
         <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K28" t="n">
-        <v>25</v>
+        <v>400</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3848,10 +3848,10 @@
         <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>29167</v>
+        <v>116667</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>3117</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>11458</v>
+        <v>45833</v>
       </c>
       <c r="K37" t="n">
-        <v>573</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>6250</v>
+        <v>25000</v>
       </c>
       <c r="K38" t="n">
-        <v>312</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K39" t="n">
-        <v>156</v>
+        <v>625</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>27083</v>
+        <v>108333</v>
       </c>
       <c r="K41" t="n">
-        <v>1354</v>
+        <v>5417</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>7292</v>
+        <v>29167</v>
       </c>
       <c r="K42" t="n">
-        <v>206</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K43" t="n">
-        <v>40</v>
+        <v>352</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1875</v>
+        <v>7500</v>
       </c>
       <c r="K44" t="n">
-        <v>88</v>
+        <v>369</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>8333</v>
+        <v>33333</v>
       </c>
       <c r="K45" t="n">
-        <v>86</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K46" t="n">
-        <v>10</v>
+        <v>791</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>308</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>30208</v>
+        <v>120833</v>
       </c>
       <c r="K49" t="n">
-        <v>294</v>
+        <v>4826</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>12500</v>
+        <v>50000</v>
       </c>
       <c r="K50" t="n">
-        <v>144</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>2708</v>
+        <v>10833</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>409</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K52" t="n">
-        <v>43</v>
+        <v>511</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>12500</v>
+        <v>50000</v>
       </c>
       <c r="K53" t="n">
-        <v>198</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>9375</v>
+        <v>37500</v>
       </c>
       <c r="K54" t="n">
-        <v>191</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K55" t="n">
-        <v>46</v>
+        <v>827</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>54167</v>
+        <v>216667</v>
       </c>
       <c r="K57" t="n">
-        <v>317</v>
+        <v>8442</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>9375</v>
+        <v>37500</v>
       </c>
       <c r="K58" t="n">
-        <v>288</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4856,10 +4856,10 @@
         <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K59" t="n">
-        <v>60</v>
+        <v>435</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>3333</v>
+        <v>13333</v>
       </c>
       <c r="K60" t="n">
-        <v>113</v>
+        <v>613</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4934,10 +4934,10 @@
         <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>8333</v>
+        <v>33333</v>
       </c>
       <c r="K61" t="n">
-        <v>78</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4973,10 +4973,10 @@
         <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K62" t="n">
-        <v>5</v>
+        <v>380</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K63" t="n">
-        <v>37</v>
+        <v>350</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>35417</v>
+        <v>141667</v>
       </c>
       <c r="K65" t="n">
-        <v>474</v>
+        <v>5787</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K66" t="n">
-        <v>260</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K67" t="n">
-        <v>104</v>
+        <v>417</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K68" t="n">
-        <v>104</v>
+        <v>417</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>7292</v>
+        <v>29167</v>
       </c>
       <c r="K69" t="n">
-        <v>365</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K70" t="n">
-        <v>125</v>
+        <v>500</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K71" t="n">
-        <v>260</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>29167</v>
+        <v>116667</v>
       </c>
       <c r="K73" t="n">
-        <v>1458</v>
+        <v>5833</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>12500</v>
+        <v>50000</v>
       </c>
       <c r="K74" t="n">
-        <v>341</v>
+        <v>2216</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>2708</v>
+        <v>10833</v>
       </c>
       <c r="K75" t="n">
-        <v>57</v>
+        <v>463</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>6250</v>
+        <v>25000</v>
       </c>
       <c r="K76" t="n">
-        <v>213</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5712,10 +5712,10 @@
         <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>31250</v>
+        <v>125000</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>4377</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>8958</v>
+        <v>35833</v>
       </c>
       <c r="K85" t="n">
-        <v>448</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>4792</v>
+        <v>19167</v>
       </c>
       <c r="K86" t="n">
-        <v>240</v>
+        <v>958</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K87" t="n">
-        <v>125</v>
+        <v>500</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>25625</v>
+        <v>102500</v>
       </c>
       <c r="K89" t="n">
-        <v>1281</v>
+        <v>5125</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>14583</v>
+        <v>58333</v>
       </c>
       <c r="K90" t="n">
-        <v>274</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K91" t="n">
-        <v>0</v>
+        <v>313</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>2500</v>
+        <v>10000</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>310</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6324,10 +6324,10 @@
         <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>31250</v>
+        <v>125000</v>
       </c>
       <c r="K97" t="n">
-        <v>293</v>
+        <v>4981</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>16667</v>
+        <v>66667</v>
       </c>
       <c r="K101" t="n">
-        <v>297</v>
+        <v>2797</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6513,10 +6513,10 @@
         <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>8333</v>
+        <v>33333</v>
       </c>
       <c r="K102" t="n">
-        <v>151</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6552,10 +6552,10 @@
         <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>5417</v>
+        <v>21667</v>
       </c>
       <c r="K103" t="n">
-        <v>0</v>
+        <v>677</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6630,10 +6630,10 @@
         <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>37500</v>
+        <v>150000</v>
       </c>
       <c r="K105" t="n">
-        <v>190</v>
+        <v>5815</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>16667</v>
+        <v>66667</v>
       </c>
       <c r="K109" t="n">
-        <v>274</v>
+        <v>2774</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6819,10 +6819,10 @@
         <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>9375</v>
+        <v>37500</v>
       </c>
       <c r="K110" t="n">
-        <v>40</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6858,10 +6858,10 @@
         <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K111" t="n">
-        <v>0</v>
+        <v>706</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6936,10 +6936,10 @@
         <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>37500</v>
+        <v>150000</v>
       </c>
       <c r="K113" t="n">
-        <v>0</v>
+        <v>5453</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6975,10 +6975,10 @@
         <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>13542</v>
+        <v>54167</v>
       </c>
       <c r="K114" t="n">
-        <v>0</v>
+        <v>1875</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7014,10 +7014,10 @@
         <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>4167</v>
+        <v>16667</v>
       </c>
       <c r="K115" t="n">
-        <v>73</v>
+        <v>698</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K116" t="n">
-        <v>29</v>
+        <v>811</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7248,10 +7248,10 @@
         <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>31250</v>
+        <v>125000</v>
       </c>
       <c r="K121" t="n">
-        <v>0</v>
+        <v>4393</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>14167</v>
+        <v>56667</v>
       </c>
       <c r="K122" t="n">
-        <v>140</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K123" t="n">
-        <v>96</v>
+        <v>565</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K124" t="n">
-        <v>51</v>
+        <v>363</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>15625</v>
+        <v>62500</v>
       </c>
       <c r="K125" t="n">
-        <v>143</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>6667</v>
+        <v>26667</v>
       </c>
       <c r="K126" t="n">
-        <v>0</v>
+        <v>783</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K127" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>58333</v>
+        <v>233333</v>
       </c>
       <c r="K129" t="n">
-        <v>193</v>
+        <v>8943</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>4167</v>
+        <v>16667</v>
       </c>
       <c r="K130" t="n">
-        <v>0</v>
+        <v>524</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K131" t="n">
-        <v>52</v>
+        <v>364</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K132" t="n">
-        <v>50</v>
+        <v>363</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>5208</v>
+        <v>20833</v>
       </c>
       <c r="K133" t="n">
-        <v>0</v>
+        <v>759</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K134" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K135" t="n">
-        <v>3</v>
+        <v>315</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>29167</v>
+        <v>116667</v>
       </c>
       <c r="K137" t="n">
-        <v>0</v>
+        <v>4187</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>4167</v>
+        <v>16667</v>
       </c>
       <c r="K138" t="n">
-        <v>0</v>
+        <v>525</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K139" t="n">
-        <v>42</v>
+        <v>354</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K140" t="n">
-        <v>92</v>
+        <v>405</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>6250</v>
+        <v>25000</v>
       </c>
       <c r="K141" t="n">
-        <v>0</v>
+        <v>912</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K142" t="n">
-        <v>21</v>
+        <v>489</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K143" t="n">
-        <v>69</v>
+        <v>537</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>31250</v>
+        <v>125000</v>
       </c>
       <c r="K145" t="n">
-        <v>215</v>
+        <v>4903</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>7292</v>
+        <v>29167</v>
       </c>
       <c r="K146" t="n">
-        <v>49</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K147" t="n">
-        <v>61</v>
+        <v>373</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>2604</v>
+        <v>10417</v>
       </c>
       <c r="K148" t="n">
-        <v>78</v>
+        <v>469</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>8333</v>
+        <v>33333</v>
       </c>
       <c r="K149" t="n">
-        <v>17</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>4167</v>
+        <v>16667</v>
       </c>
       <c r="K150" t="n">
-        <v>0</v>
+        <v>601</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>3125</v>
+        <v>12500</v>
       </c>
       <c r="K151" t="n">
-        <v>0</v>
+        <v>460</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>31250</v>
+        <v>125000</v>
       </c>
       <c r="K153" t="n">
-        <v>0</v>
+        <v>4586</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>6250</v>
+        <v>25000</v>
       </c>
       <c r="K154" t="n">
-        <v>13</v>
+        <v>950</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8588,10 +8588,10 @@
         <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K155" t="n">
-        <v>5</v>
+        <v>318</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8627,10 +8627,10 @@
         <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>2083</v>
+        <v>8333</v>
       </c>
       <c r="K156" t="n">
-        <v>0</v>
+        <v>306</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>25000</v>
+        <v>100000</v>
       </c>
       <c r="K161" t="n">
-        <v>0</v>
+        <v>3160</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>13542</v>
+        <v>54167</v>
       </c>
       <c r="K165" t="n">
-        <v>677</v>
+        <v>2708</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>7917</v>
+        <v>31667</v>
       </c>
       <c r="K166" t="n">
-        <v>396</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>5833</v>
+        <v>23333</v>
       </c>
       <c r="K167" t="n">
-        <v>292</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>34792</v>
+        <v>139167</v>
       </c>
       <c r="K169" t="n">
-        <v>1740</v>
+        <v>6958</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9167,10 +9167,10 @@
         <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>155208</v>
+        <v>620833</v>
       </c>
       <c r="K170" t="n">
-        <v>6758</v>
+        <v>30039</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9206,10 +9206,10 @@
         <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>37500</v>
+        <v>150000</v>
       </c>
       <c r="K171" t="n">
-        <v>236</v>
+        <v>5861</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9245,10 +9245,10 @@
         <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>28125</v>
+        <v>112500</v>
       </c>
       <c r="K172" t="n">
-        <v>1276</v>
+        <v>5494</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>385417</v>
+        <v>1541667</v>
       </c>
       <c r="K173" t="n">
-        <v>17532</v>
+        <v>75345</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9323,10 +9323,10 @@
         <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>19792</v>
+        <v>79167</v>
       </c>
       <c r="K174" t="n">
-        <v>201</v>
+        <v>3170</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>19792</v>
+        <v>79167</v>
       </c>
       <c r="K175" t="n">
-        <v>710</v>
+        <v>3679</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>887500</v>
+        <v>3550000</v>
       </c>
       <c r="K177" t="n">
-        <v>31855</v>
+        <v>164980</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9479,10 +9479,10 @@
         <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>66667</v>
+        <v>266667</v>
       </c>
       <c r="K178" t="n">
-        <v>1236</v>
+        <v>11236</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9518,10 +9518,10 @@
         <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>16667</v>
+        <v>66667</v>
       </c>
       <c r="K179" t="n">
-        <v>286</v>
+        <v>2786</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9557,10 +9557,10 @@
         <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>24167</v>
+        <v>96667</v>
       </c>
       <c r="K180" t="n">
-        <v>775</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9596,10 +9596,10 @@
         <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>66250</v>
+        <v>265000</v>
       </c>
       <c r="K181" t="n">
-        <v>690</v>
+        <v>10628</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>37917</v>
+        <v>151667</v>
       </c>
       <c r="K182" t="n">
-        <v>349</v>
+        <v>6036</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>22708</v>
+        <v>90833</v>
       </c>
       <c r="K183" t="n">
-        <v>240</v>
+        <v>3647</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>315208</v>
+        <v>1260833</v>
       </c>
       <c r="K185" t="n">
-        <v>3846</v>
+        <v>51127</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>1550000</v>
+        <v>6200000</v>
       </c>
       <c r="K187" t="n">
-        <v>36986</v>
+        <v>269486</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>750000</v>
+        <v>3000000</v>
       </c>
       <c r="K188" t="n">
-        <v>21465</v>
+        <v>133965</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>791667</v>
+        <v>3166667</v>
       </c>
       <c r="K189" t="n">
-        <v>21624</v>
+        <v>140374</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">

</xml_diff>

<commit_message>
feat(visites): add drag-drop preview, atomic save, heure fin and tournee names in date filter
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2961,10 +2961,10 @@
         <v>4831</v>
       </c>
       <c r="J10" t="n">
-        <v>37500</v>
+        <v>45000</v>
       </c>
       <c r="K10" t="n">
-        <v>1399</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3000,10 +3000,10 @@
         <v>534</v>
       </c>
       <c r="J11" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K11" t="n">
-        <v>438</v>
+        <v>717</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3039,10 +3039,10 @@
         <v>-82</v>
       </c>
       <c r="J12" t="n">
-        <v>20000</v>
+        <v>24000</v>
       </c>
       <c r="K12" t="n">
-        <v>939</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3230,10 +3230,10 @@
         <v>10255</v>
       </c>
       <c r="J17" t="n">
-        <v>108333</v>
+        <v>130000</v>
       </c>
       <c r="K17" t="n">
-        <v>4341</v>
+        <v>7232</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3380,10 +3380,10 @@
         <v>4641</v>
       </c>
       <c r="J21" t="n">
-        <v>37500</v>
+        <v>45000</v>
       </c>
       <c r="K21" t="n">
-        <v>1404</v>
+        <v>2372</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3419,10 +3419,10 @@
         <v>2704</v>
       </c>
       <c r="J22" t="n">
-        <v>29167</v>
+        <v>35000</v>
       </c>
       <c r="K22" t="n">
-        <v>1122</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3458,10 +3458,10 @@
         <v>1756</v>
       </c>
       <c r="J23" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K23" t="n">
-        <v>347</v>
+        <v>596</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3536,10 +3536,10 @@
         <v>13570</v>
       </c>
       <c r="J25" t="n">
-        <v>104167</v>
+        <v>125000</v>
       </c>
       <c r="K25" t="n">
-        <v>3864</v>
+        <v>6541</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3575,10 +3575,10 @@
         <v>3178</v>
       </c>
       <c r="J26" t="n">
-        <v>41667</v>
+        <v>50000</v>
       </c>
       <c r="K26" t="n">
-        <v>1567</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3614,10 +3614,10 @@
         <v>928</v>
       </c>
       <c r="J27" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K27" t="n">
-        <v>272</v>
+        <v>474</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3653,10 +3653,10 @@
         <v>282</v>
       </c>
       <c r="J28" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K28" t="n">
-        <v>400</v>
+        <v>667</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3848,10 +3848,10 @@
         <v>14696</v>
       </c>
       <c r="J33" t="n">
-        <v>116667</v>
+        <v>140000</v>
       </c>
       <c r="K33" t="n">
-        <v>3117</v>
+        <v>5711</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>45833</v>
+        <v>55000</v>
       </c>
       <c r="K37" t="n">
-        <v>2292</v>
+        <v>3667</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4037,10 +4037,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="K38" t="n">
-        <v>1250</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4076,10 +4076,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K39" t="n">
-        <v>625</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4154,10 +4154,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>108333</v>
+        <v>130000</v>
       </c>
       <c r="K41" t="n">
-        <v>5417</v>
+        <v>8667</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4193,10 +4193,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>29167</v>
+        <v>35000</v>
       </c>
       <c r="K42" t="n">
-        <v>1300</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4232,10 +4232,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K43" t="n">
-        <v>352</v>
+        <v>581</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4271,10 +4271,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>7500</v>
+        <v>9000</v>
       </c>
       <c r="K44" t="n">
-        <v>369</v>
+        <v>592</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4310,10 +4310,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>33333</v>
+        <v>40000</v>
       </c>
       <c r="K45" t="n">
-        <v>1336</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4349,10 +4349,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K46" t="n">
-        <v>791</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4388,10 +4388,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K47" t="n">
-        <v>308</v>
+        <v>521</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4466,10 +4466,10 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>120833</v>
+        <v>145000</v>
       </c>
       <c r="K49" t="n">
-        <v>4826</v>
+        <v>8045</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4505,10 +4505,10 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="K50" t="n">
-        <v>2019</v>
+        <v>3359</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>10833</v>
+        <v>13000</v>
       </c>
       <c r="K51" t="n">
-        <v>409</v>
+        <v>690</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4583,10 +4583,10 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K52" t="n">
-        <v>511</v>
+        <v>848</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4622,10 +4622,10 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="K53" t="n">
-        <v>2073</v>
+        <v>3431</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>37500</v>
+        <v>45000</v>
       </c>
       <c r="K54" t="n">
-        <v>1597</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4700,10 +4700,10 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K55" t="n">
-        <v>827</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4778,10 +4778,10 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>216667</v>
+        <v>260000</v>
       </c>
       <c r="K57" t="n">
-        <v>8442</v>
+        <v>14144</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4817,10 +4817,10 @@
         <v>545</v>
       </c>
       <c r="J58" t="n">
-        <v>37500</v>
+        <v>45000</v>
       </c>
       <c r="K58" t="n">
-        <v>1694</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4856,10 +4856,10 @@
         <v>101</v>
       </c>
       <c r="J59" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K59" t="n">
-        <v>435</v>
+        <v>713</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4895,10 +4895,10 @@
         <v>190</v>
       </c>
       <c r="J60" t="n">
-        <v>13333</v>
+        <v>16000</v>
       </c>
       <c r="K60" t="n">
-        <v>613</v>
+        <v>995</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4934,10 +4934,10 @@
         <v>974</v>
       </c>
       <c r="J61" t="n">
-        <v>33333</v>
+        <v>40000</v>
       </c>
       <c r="K61" t="n">
-        <v>1328</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4973,10 +4973,10 @@
         <v>1009</v>
       </c>
       <c r="J62" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K62" t="n">
-        <v>380</v>
+        <v>639</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5012,10 +5012,10 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K63" t="n">
-        <v>350</v>
+        <v>578</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5090,10 +5090,10 @@
         <v>4972</v>
       </c>
       <c r="J65" t="n">
-        <v>141667</v>
+        <v>170000</v>
       </c>
       <c r="K65" t="n">
-        <v>5787</v>
+        <v>9605</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5129,10 +5129,10 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K66" t="n">
-        <v>1042</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5168,10 +5168,10 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K67" t="n">
-        <v>417</v>
+        <v>667</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5207,10 +5207,10 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K68" t="n">
-        <v>417</v>
+        <v>667</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5246,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>29167</v>
+        <v>35000</v>
       </c>
       <c r="K69" t="n">
-        <v>1458</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5285,10 +5285,10 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K70" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5324,10 +5324,10 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K71" t="n">
-        <v>1042</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>116667</v>
+        <v>140000</v>
       </c>
       <c r="K73" t="n">
-        <v>5833</v>
+        <v>9333</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5441,10 +5441,10 @@
         <v>1835</v>
       </c>
       <c r="J74" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="K74" t="n">
-        <v>2216</v>
+        <v>3621</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5480,10 +5480,10 @@
         <v>605</v>
       </c>
       <c r="J75" t="n">
-        <v>10833</v>
+        <v>13000</v>
       </c>
       <c r="K75" t="n">
-        <v>463</v>
+        <v>762</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5519,10 +5519,10 @@
         <v>520</v>
       </c>
       <c r="J76" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="K76" t="n">
-        <v>1151</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5712,10 +5712,10 @@
         <v>15733</v>
       </c>
       <c r="J81" t="n">
-        <v>125000</v>
+        <v>150000</v>
       </c>
       <c r="K81" t="n">
-        <v>4377</v>
+        <v>7502</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5862,10 +5862,10 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>35833</v>
+        <v>43000</v>
       </c>
       <c r="K85" t="n">
-        <v>1792</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5901,10 +5901,10 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>19167</v>
+        <v>23000</v>
       </c>
       <c r="K86" t="n">
-        <v>958</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5940,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K87" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6018,10 +6018,10 @@
         <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>102500</v>
+        <v>123000</v>
       </c>
       <c r="K89" t="n">
-        <v>5125</v>
+        <v>8200</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6057,10 +6057,10 @@
         <v>2168</v>
       </c>
       <c r="J90" t="n">
-        <v>58333</v>
+        <v>70000</v>
       </c>
       <c r="K90" t="n">
-        <v>2462</v>
+        <v>4060</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6096,10 +6096,10 @@
         <v>403</v>
       </c>
       <c r="J91" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K91" t="n">
-        <v>313</v>
+        <v>528</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6135,10 +6135,10 @@
         <v>1200</v>
       </c>
       <c r="J92" t="n">
-        <v>10000</v>
+        <v>12000</v>
       </c>
       <c r="K92" t="n">
-        <v>310</v>
+        <v>547</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6324,10 +6324,10 @@
         <v>6326</v>
       </c>
       <c r="J97" t="n">
-        <v>125000</v>
+        <v>150000</v>
       </c>
       <c r="K97" t="n">
-        <v>4981</v>
+        <v>8307</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6474,10 +6474,10 @@
         <v>3414</v>
       </c>
       <c r="J101" t="n">
-        <v>66667</v>
+        <v>80000</v>
       </c>
       <c r="K101" t="n">
-        <v>2797</v>
+        <v>4618</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6513,10 +6513,10 @@
         <v>1244</v>
       </c>
       <c r="J102" t="n">
-        <v>33333</v>
+        <v>40000</v>
       </c>
       <c r="K102" t="n">
-        <v>1401</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6552,10 +6552,10 @@
         <v>1781</v>
       </c>
       <c r="J103" t="n">
-        <v>21667</v>
+        <v>26000</v>
       </c>
       <c r="K103" t="n">
-        <v>677</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6630,10 +6630,10 @@
         <v>9207</v>
       </c>
       <c r="J105" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="K105" t="n">
-        <v>5815</v>
+        <v>9754</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6780,10 +6780,10 @@
         <v>1240</v>
       </c>
       <c r="J109" t="n">
-        <v>66667</v>
+        <v>80000</v>
       </c>
       <c r="K109" t="n">
-        <v>2774</v>
+        <v>4587</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6819,10 +6819,10 @@
         <v>815</v>
       </c>
       <c r="J110" t="n">
-        <v>37500</v>
+        <v>45000</v>
       </c>
       <c r="K110" t="n">
-        <v>1446</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6858,10 +6858,10 @@
         <v>628</v>
       </c>
       <c r="J111" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K111" t="n">
-        <v>706</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6936,10 +6936,10 @@
         <v>5380</v>
       </c>
       <c r="J113" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="K113" t="n">
-        <v>5453</v>
+        <v>9270</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6975,10 +6975,10 @@
         <v>3030</v>
       </c>
       <c r="J114" t="n">
-        <v>54167</v>
+        <v>65000</v>
       </c>
       <c r="K114" t="n">
-        <v>1875</v>
+        <v>3223</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7014,10 +7014,10 @@
         <v>817</v>
       </c>
       <c r="J115" t="n">
-        <v>16667</v>
+        <v>20000</v>
       </c>
       <c r="K115" t="n">
-        <v>698</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7053,10 +7053,10 @@
         <v>641</v>
       </c>
       <c r="J116" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K116" t="n">
-        <v>811</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7248,10 +7248,10 @@
         <v>6773</v>
       </c>
       <c r="J121" t="n">
-        <v>125000</v>
+        <v>150000</v>
       </c>
       <c r="K121" t="n">
-        <v>4393</v>
+        <v>7524</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7287,10 +7287,10 @@
         <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>56667</v>
+        <v>68000</v>
       </c>
       <c r="K122" t="n">
-        <v>2265</v>
+        <v>3775</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K123" t="n">
-        <v>565</v>
+        <v>920</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7365,10 +7365,10 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K124" t="n">
-        <v>363</v>
+        <v>596</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7404,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>62500</v>
+        <v>75000</v>
       </c>
       <c r="K125" t="n">
-        <v>2487</v>
+        <v>4149</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7443,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>26667</v>
+        <v>32000</v>
       </c>
       <c r="K126" t="n">
-        <v>783</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7482,10 +7482,10 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K127" t="n">
-        <v>312</v>
+        <v>528</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7560,10 +7560,10 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>233333</v>
+        <v>280000</v>
       </c>
       <c r="K129" t="n">
-        <v>8943</v>
+        <v>15035</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>16667</v>
+        <v>20000</v>
       </c>
       <c r="K130" t="n">
-        <v>524</v>
+        <v>921</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7642,10 +7642,10 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K131" t="n">
-        <v>364</v>
+        <v>597</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K132" t="n">
-        <v>363</v>
+        <v>595</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7724,10 +7724,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>20833</v>
+        <v>25000</v>
       </c>
       <c r="K133" t="n">
-        <v>759</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7765,10 +7765,10 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K134" t="n">
-        <v>410</v>
+        <v>713</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7806,10 +7806,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K135" t="n">
-        <v>315</v>
+        <v>531</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7886,10 +7886,10 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>116667</v>
+        <v>140000</v>
       </c>
       <c r="K137" t="n">
-        <v>4187</v>
+        <v>7138</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>16667</v>
+        <v>20000</v>
       </c>
       <c r="K138" t="n">
-        <v>525</v>
+        <v>923</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7964,10 +7964,10 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K139" t="n">
-        <v>354</v>
+        <v>583</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8003,10 +8003,10 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K140" t="n">
-        <v>405</v>
+        <v>651</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8042,10 +8042,10 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="K141" t="n">
-        <v>912</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8081,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="J142" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K142" t="n">
-        <v>489</v>
+        <v>819</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8120,10 +8120,10 @@
         <v>0</v>
       </c>
       <c r="J143" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K143" t="n">
-        <v>537</v>
+        <v>883</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8198,10 +8198,10 @@
         <v>0</v>
       </c>
       <c r="J145" t="n">
-        <v>125000</v>
+        <v>150000</v>
       </c>
       <c r="K145" t="n">
-        <v>4903</v>
+        <v>8204</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>29167</v>
+        <v>35000</v>
       </c>
       <c r="K146" t="n">
-        <v>1143</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8276,10 +8276,10 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K147" t="n">
-        <v>373</v>
+        <v>609</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8315,10 +8315,10 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>10417</v>
+        <v>12500</v>
       </c>
       <c r="K148" t="n">
-        <v>469</v>
+        <v>764</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8354,10 +8354,10 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>33333</v>
+        <v>40000</v>
       </c>
       <c r="K149" t="n">
-        <v>1267</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8393,10 +8393,10 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>16667</v>
+        <v>20000</v>
       </c>
       <c r="K150" t="n">
-        <v>601</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8432,10 +8432,10 @@
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>12500</v>
+        <v>15000</v>
       </c>
       <c r="K151" t="n">
-        <v>460</v>
+        <v>780</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8510,10 +8510,10 @@
         <v>0</v>
       </c>
       <c r="J153" t="n">
-        <v>125000</v>
+        <v>150000</v>
       </c>
       <c r="K153" t="n">
-        <v>4586</v>
+        <v>7781</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8549,10 +8549,10 @@
         <v>2380</v>
       </c>
       <c r="J154" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="K154" t="n">
-        <v>950</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8588,10 +8588,10 @@
         <v>1190</v>
       </c>
       <c r="J155" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K155" t="n">
-        <v>318</v>
+        <v>535</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8627,10 +8627,10 @@
         <v>22</v>
       </c>
       <c r="J156" t="n">
-        <v>8333</v>
+        <v>10000</v>
       </c>
       <c r="K156" t="n">
-        <v>306</v>
+        <v>519</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8822,10 +8822,10 @@
         <v>8836</v>
       </c>
       <c r="J161" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="K161" t="n">
-        <v>3160</v>
+        <v>5546</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8972,10 +8972,10 @@
         <v>0</v>
       </c>
       <c r="J165" t="n">
-        <v>54167</v>
+        <v>65000</v>
       </c>
       <c r="K165" t="n">
-        <v>2708</v>
+        <v>4333</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9011,10 +9011,10 @@
         <v>0</v>
       </c>
       <c r="J166" t="n">
-        <v>31667</v>
+        <v>38000</v>
       </c>
       <c r="K166" t="n">
-        <v>1583</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9050,10 +9050,10 @@
         <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>23333</v>
+        <v>28000</v>
       </c>
       <c r="K167" t="n">
-        <v>1167</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9128,10 +9128,10 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>139167</v>
+        <v>167000</v>
       </c>
       <c r="K169" t="n">
-        <v>6958</v>
+        <v>11133</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9167,10 +9167,10 @@
         <v>6510</v>
       </c>
       <c r="J170" t="n">
-        <v>620833</v>
+        <v>745000</v>
       </c>
       <c r="K170" t="n">
-        <v>30039</v>
+        <v>48330</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9206,10 +9206,10 @@
         <v>12899</v>
       </c>
       <c r="J171" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="K171" t="n">
-        <v>5861</v>
+        <v>9814</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9245,10 +9245,10 @@
         <v>2129</v>
       </c>
       <c r="J172" t="n">
-        <v>112500</v>
+        <v>135000</v>
       </c>
       <c r="K172" t="n">
-        <v>5494</v>
+        <v>8826</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9284,10 +9284,10 @@
         <v>21357</v>
       </c>
       <c r="J173" t="n">
-        <v>1541667</v>
+        <v>1850000</v>
       </c>
       <c r="K173" t="n">
-        <v>75345</v>
+        <v>121015</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9323,10 +9323,10 @@
         <v>3801</v>
       </c>
       <c r="J174" t="n">
-        <v>79167</v>
+        <v>95000</v>
       </c>
       <c r="K174" t="n">
-        <v>3170</v>
+        <v>5282</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9362,10 +9362,10 @@
         <v>4149</v>
       </c>
       <c r="J175" t="n">
-        <v>79167</v>
+        <v>95000</v>
       </c>
       <c r="K175" t="n">
-        <v>3679</v>
+        <v>5960</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9440,10 +9440,10 @@
         <v>123920</v>
       </c>
       <c r="J177" t="n">
-        <v>3550000</v>
+        <v>4260000</v>
       </c>
       <c r="K177" t="n">
-        <v>164980</v>
+        <v>267307</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9479,10 +9479,10 @@
         <v>10389</v>
       </c>
       <c r="J178" t="n">
-        <v>266667</v>
+        <v>320000</v>
       </c>
       <c r="K178" t="n">
-        <v>11236</v>
+        <v>18537</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9518,10 +9518,10 @@
         <v>2168</v>
       </c>
       <c r="J179" t="n">
-        <v>66667</v>
+        <v>80000</v>
       </c>
       <c r="K179" t="n">
-        <v>2786</v>
+        <v>4604</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9557,10 +9557,10 @@
         <v>910</v>
       </c>
       <c r="J180" t="n">
-        <v>96667</v>
+        <v>116000</v>
       </c>
       <c r="K180" t="n">
-        <v>4400</v>
+        <v>7156</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9596,10 +9596,10 @@
         <v>11859</v>
       </c>
       <c r="J181" t="n">
-        <v>265000</v>
+        <v>318000</v>
       </c>
       <c r="K181" t="n">
-        <v>10628</v>
+        <v>17704</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9635,10 +9635,10 @@
         <v>7489</v>
       </c>
       <c r="J182" t="n">
-        <v>151667</v>
+        <v>182000</v>
       </c>
       <c r="K182" t="n">
-        <v>6036</v>
+        <v>10070</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9674,10 +9674,10 @@
         <v>2004</v>
       </c>
       <c r="J183" t="n">
-        <v>90833</v>
+        <v>109000</v>
       </c>
       <c r="K183" t="n">
-        <v>3647</v>
+        <v>6073</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9752,10 +9752,10 @@
         <v>59226</v>
       </c>
       <c r="J185" t="n">
-        <v>1260833</v>
+        <v>1513000</v>
       </c>
       <c r="K185" t="n">
-        <v>51127</v>
+        <v>84981</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9830,10 +9830,10 @@
         <v>219668</v>
       </c>
       <c r="J187" t="n">
-        <v>6200000</v>
+        <v>7440000</v>
       </c>
       <c r="K187" t="n">
-        <v>269486</v>
+        <v>441982</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9869,10 +9869,10 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>3000000</v>
+        <v>3600000</v>
       </c>
       <c r="K188" t="n">
-        <v>133965</v>
+        <v>218620</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9908,10 +9908,10 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>3166667</v>
+        <v>3800000</v>
       </c>
       <c r="K189" t="n">
-        <v>140374</v>
+        <v>229387</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">
@@ -10221,10 +10221,10 @@
         <v>0.159622112638379</v>
       </c>
       <c r="H2" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -10252,10 +10252,10 @@
         <v>0.13006246214979</v>
       </c>
       <c r="H3" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I3" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="250">
@@ -10283,10 +10283,10 @@
         <v>0.12785218855059</v>
       </c>
       <c r="H4" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I4" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="250">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="G5" s="258" t="n"/>
       <c r="I5" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="250">
@@ -10338,10 +10338,10 @@
         <v>0.119182965859955</v>
       </c>
       <c r="H6" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="I6" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="250" thickBot="1">
@@ -10369,10 +10369,10 @@
         <v>0.106909295617267</v>
       </c>
       <c r="H7" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="I7" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="158">
@@ -10400,10 +10400,10 @@
         <v>0.127185196510197</v>
       </c>
       <c r="H8" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I8" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="250">
@@ -10431,10 +10431,10 @@
         <v>0.130798384540069</v>
       </c>
       <c r="H9" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I9" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="250">
@@ -10462,10 +10462,10 @@
         <v>0.197218920214015</v>
       </c>
       <c r="H10" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I10" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="250">
@@ -10493,10 +10493,10 @@
         <v>0.156143076621019</v>
       </c>
       <c r="H11" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I11" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="250">
@@ -10524,10 +10524,10 @@
         <v>0.125550416455854</v>
       </c>
       <c r="H12" t="n">
-        <v>229</v>
+        <v>305</v>
       </c>
       <c r="I12" t="n">
-        <v>207</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="250">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="G13" s="258" t="n"/>
       <c r="I13" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="250">
@@ -10579,10 +10579,10 @@
         <v>0.0806766817717267</v>
       </c>
       <c r="H14" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="I14" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="250">
@@ -10610,10 +10610,10 @@
         <v>0.0777021675916213</v>
       </c>
       <c r="H15" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="I15" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="250">
@@ -10637,7 +10637,7 @@
       </c>
       <c r="G16" s="260" t="n"/>
       <c r="I16" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="250">
@@ -10665,10 +10665,10 @@
         <v>0.095303991140541</v>
       </c>
       <c r="H17" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I17" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="250">
@@ -10696,10 +10696,10 @@
         <v>0.0776551038922926</v>
       </c>
       <c r="H18" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="I18" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="250">
@@ -10727,10 +10727,10 @@
         <v>0.162114464314885</v>
       </c>
       <c r="H19" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="I19" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="250">
@@ -10754,7 +10754,7 @@
       </c>
       <c r="G20" s="208" t="n"/>
       <c r="I20" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="250">
@@ -10782,10 +10782,10 @@
         <v>0.08919891687813671</v>
       </c>
       <c r="H21" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="I21" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="250">
@@ -10813,10 +10813,10 @@
         <v>0.08301513631583469</v>
       </c>
       <c r="H22" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="I22" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="250">
@@ -10844,10 +10844,10 @@
         <v>0.06665486782805979</v>
       </c>
       <c r="H23" t="n">
-        <v>286</v>
+        <v>381</v>
       </c>
       <c r="I23" t="n">
-        <v>271</v>
+        <v>362</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="250">
@@ -10875,10 +10875,10 @@
         <v>0.07487484353666519</v>
       </c>
       <c r="H24" t="n">
-        <v>551</v>
+        <v>734</v>
       </c>
       <c r="I24" t="n">
-        <v>508</v>
+        <v>677</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="250">

</xml_diff>

<commit_message>
feat: add historique snapshot system, WhatsApp focus links, Theme 6, and Vercel handler
</commit_message>
<xml_diff>
--- a/excel/finale_jour.xlsx
+++ b/excel/finale_jour.xlsx
@@ -2964,7 +2964,7 @@
         <v>45000</v>
       </c>
       <c r="K10" t="n">
-        <v>2366</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="250">
@@ -3003,7 +3003,7 @@
         <v>12000</v>
       </c>
       <c r="K11" t="n">
-        <v>717</v>
+        <v>566</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="250">
@@ -3042,7 +3042,7 @@
         <v>24000</v>
       </c>
       <c r="K12" t="n">
-        <v>1519</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="250">
@@ -3233,7 +3233,7 @@
         <v>130000</v>
       </c>
       <c r="K17" t="n">
-        <v>7232</v>
+        <v>5710</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1" s="250">
@@ -3383,7 +3383,7 @@
         <v>45000</v>
       </c>
       <c r="K21" t="n">
-        <v>2372</v>
+        <v>1873</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="250">
@@ -3422,7 +3422,7 @@
         <v>35000</v>
       </c>
       <c r="K22" t="n">
-        <v>1884</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1" s="250">
@@ -3461,7 +3461,7 @@
         <v>12000</v>
       </c>
       <c r="K23" t="n">
-        <v>596</v>
+        <v>471</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1" s="250">
@@ -3539,7 +3539,7 @@
         <v>125000</v>
       </c>
       <c r="K25" t="n">
-        <v>6541</v>
+        <v>5164</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="250">
@@ -3578,7 +3578,7 @@
         <v>50000</v>
       </c>
       <c r="K26" t="n">
-        <v>2645</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1" s="250">
@@ -3617,7 +3617,7 @@
         <v>10000</v>
       </c>
       <c r="K27" t="n">
-        <v>474</v>
+        <v>375</v>
       </c>
     </row>
     <row r="28" ht="14.25" customHeight="1" s="250">
@@ -3656,7 +3656,7 @@
         <v>12000</v>
       </c>
       <c r="K28" t="n">
-        <v>667</v>
+        <v>526</v>
       </c>
     </row>
     <row r="29" ht="14.25" customHeight="1" s="250">
@@ -3851,7 +3851,7 @@
         <v>140000</v>
       </c>
       <c r="K33" t="n">
-        <v>5711</v>
+        <v>4509</v>
       </c>
     </row>
     <row r="34" ht="14.25" customHeight="1" s="250">
@@ -4001,7 +4001,7 @@
         <v>55000</v>
       </c>
       <c r="K37" t="n">
-        <v>3667</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="250">
@@ -4040,7 +4040,7 @@
         <v>30000</v>
       </c>
       <c r="K38" t="n">
-        <v>2000</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="250">
@@ -4079,7 +4079,7 @@
         <v>15000</v>
       </c>
       <c r="K39" t="n">
-        <v>1000</v>
+        <v>789</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" s="250">
@@ -4157,7 +4157,7 @@
         <v>130000</v>
       </c>
       <c r="K41" t="n">
-        <v>8667</v>
+        <v>6842</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1" s="250">
@@ -4196,7 +4196,7 @@
         <v>35000</v>
       </c>
       <c r="K42" t="n">
-        <v>2122</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="43" ht="14.25" customHeight="1" s="250">
@@ -4235,7 +4235,7 @@
         <v>10000</v>
       </c>
       <c r="K43" t="n">
-        <v>581</v>
+        <v>458</v>
       </c>
     </row>
     <row r="44" ht="14.25" customHeight="1" s="250">
@@ -4274,7 +4274,7 @@
         <v>9000</v>
       </c>
       <c r="K44" t="n">
-        <v>592</v>
+        <v>467</v>
       </c>
     </row>
     <row r="45" ht="14.25" customHeight="1" s="250">
@@ -4313,7 +4313,7 @@
         <v>40000</v>
       </c>
       <c r="K45" t="n">
-        <v>2225</v>
+        <v>1757</v>
       </c>
     </row>
     <row r="46" ht="14.25" customHeight="1" s="250">
@@ -4352,7 +4352,7 @@
         <v>25000</v>
       </c>
       <c r="K46" t="n">
-        <v>1332</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="47" ht="14.25" customHeight="1" s="250">
@@ -4391,7 +4391,7 @@
         <v>10000</v>
       </c>
       <c r="K47" t="n">
-        <v>521</v>
+        <v>412</v>
       </c>
     </row>
     <row r="48" ht="14.25" customHeight="1" s="250">
@@ -4469,7 +4469,7 @@
         <v>145000</v>
       </c>
       <c r="K49" t="n">
-        <v>8045</v>
+        <v>6352</v>
       </c>
     </row>
     <row r="50" ht="14.25" customHeight="1" s="250">
@@ -4508,7 +4508,7 @@
         <v>60000</v>
       </c>
       <c r="K50" t="n">
-        <v>3359</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="51" ht="14.25" customHeight="1" s="250">
@@ -4547,7 +4547,7 @@
         <v>13000</v>
       </c>
       <c r="K51" t="n">
-        <v>690</v>
+        <v>545</v>
       </c>
     </row>
     <row r="52" ht="14.25" customHeight="1" s="250">
@@ -4586,7 +4586,7 @@
         <v>15000</v>
       </c>
       <c r="K52" t="n">
-        <v>848</v>
+        <v>670</v>
       </c>
     </row>
     <row r="53" ht="14.25" customHeight="1" s="250">
@@ -4625,7 +4625,7 @@
         <v>60000</v>
       </c>
       <c r="K53" t="n">
-        <v>3431</v>
+        <v>2709</v>
       </c>
     </row>
     <row r="54" ht="14.25" customHeight="1" s="250">
@@ -4664,7 +4664,7 @@
         <v>45000</v>
       </c>
       <c r="K54" t="n">
-        <v>2629</v>
+        <v>2076</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1" s="250">
@@ -4703,7 +4703,7 @@
         <v>25000</v>
       </c>
       <c r="K55" t="n">
-        <v>1381</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="56" ht="14.25" customHeight="1" s="250">
@@ -4781,7 +4781,7 @@
         <v>260000</v>
       </c>
       <c r="K57" t="n">
-        <v>14144</v>
+        <v>11167</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1" s="250">
@@ -4820,7 +4820,7 @@
         <v>45000</v>
       </c>
       <c r="K58" t="n">
-        <v>2758</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1" s="250">
@@ -4859,7 +4859,7 @@
         <v>12000</v>
       </c>
       <c r="K59" t="n">
-        <v>713</v>
+        <v>563</v>
       </c>
     </row>
     <row r="60" ht="14.25" customHeight="1" s="250">
@@ -4898,7 +4898,7 @@
         <v>16000</v>
       </c>
       <c r="K60" t="n">
-        <v>995</v>
+        <v>786</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1" s="250">
@@ -4937,7 +4937,7 @@
         <v>40000</v>
       </c>
       <c r="K61" t="n">
-        <v>2215</v>
+        <v>1748</v>
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1" s="250">
@@ -4976,7 +4976,7 @@
         <v>12000</v>
       </c>
       <c r="K62" t="n">
-        <v>639</v>
+        <v>505</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1" s="250">
@@ -5015,7 +5015,7 @@
         <v>10000</v>
       </c>
       <c r="K63" t="n">
-        <v>578</v>
+        <v>456</v>
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1" s="250">
@@ -5093,7 +5093,7 @@
         <v>170000</v>
       </c>
       <c r="K65" t="n">
-        <v>9605</v>
+        <v>7583</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1" s="250">
@@ -5132,7 +5132,7 @@
         <v>25000</v>
       </c>
       <c r="K66" t="n">
-        <v>1667</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="67" ht="14.25" customHeight="1" s="250">
@@ -5171,7 +5171,7 @@
         <v>10000</v>
       </c>
       <c r="K67" t="n">
-        <v>667</v>
+        <v>526</v>
       </c>
     </row>
     <row r="68" ht="14.25" customHeight="1" s="250">
@@ -5210,7 +5210,7 @@
         <v>10000</v>
       </c>
       <c r="K68" t="n">
-        <v>667</v>
+        <v>526</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1" s="250">
@@ -5249,7 +5249,7 @@
         <v>35000</v>
       </c>
       <c r="K69" t="n">
-        <v>2333</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1" s="250">
@@ -5288,7 +5288,7 @@
         <v>12000</v>
       </c>
       <c r="K70" t="n">
-        <v>800</v>
+        <v>632</v>
       </c>
     </row>
     <row r="71" ht="14.25" customHeight="1" s="250">
@@ -5327,7 +5327,7 @@
         <v>25000</v>
       </c>
       <c r="K71" t="n">
-        <v>1667</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="72" ht="14.25" customHeight="1" s="250">
@@ -5405,7 +5405,7 @@
         <v>140000</v>
       </c>
       <c r="K73" t="n">
-        <v>9333</v>
+        <v>7368</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1" s="250">
@@ -5444,7 +5444,7 @@
         <v>60000</v>
       </c>
       <c r="K74" t="n">
-        <v>3621</v>
+        <v>2858</v>
       </c>
     </row>
     <row r="75" ht="14.25" customHeight="1" s="250">
@@ -5483,7 +5483,7 @@
         <v>13000</v>
       </c>
       <c r="K75" t="n">
-        <v>762</v>
+        <v>601</v>
       </c>
     </row>
     <row r="76" ht="14.25" customHeight="1" s="250">
@@ -5522,7 +5522,7 @@
         <v>30000</v>
       </c>
       <c r="K76" t="n">
-        <v>1868</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="77" ht="14.25" customHeight="1" s="250">
@@ -5715,7 +5715,7 @@
         <v>150000</v>
       </c>
       <c r="K81" t="n">
-        <v>7502</v>
+        <v>5923</v>
       </c>
     </row>
     <row r="82" ht="14.25" customHeight="1" s="250">
@@ -5865,7 +5865,7 @@
         <v>43000</v>
       </c>
       <c r="K85" t="n">
-        <v>2867</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="86" ht="14.25" customHeight="1" s="250">
@@ -5904,7 +5904,7 @@
         <v>23000</v>
       </c>
       <c r="K86" t="n">
-        <v>1533</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="87" ht="14.25" customHeight="1" s="250">
@@ -5943,7 +5943,7 @@
         <v>12000</v>
       </c>
       <c r="K87" t="n">
-        <v>800</v>
+        <v>632</v>
       </c>
     </row>
     <row r="88" ht="14.25" customHeight="1" s="250">
@@ -6021,7 +6021,7 @@
         <v>123000</v>
       </c>
       <c r="K89" t="n">
-        <v>8200</v>
+        <v>6474</v>
       </c>
     </row>
     <row r="90" ht="14.25" customHeight="1" s="250">
@@ -6060,7 +6060,7 @@
         <v>70000</v>
       </c>
       <c r="K90" t="n">
-        <v>4060</v>
+        <v>3205</v>
       </c>
     </row>
     <row r="91" ht="14.25" customHeight="1" s="250">
@@ -6099,7 +6099,7 @@
         <v>10000</v>
       </c>
       <c r="K91" t="n">
-        <v>528</v>
+        <v>417</v>
       </c>
     </row>
     <row r="92" ht="14.25" customHeight="1" s="250">
@@ -6138,7 +6138,7 @@
         <v>12000</v>
       </c>
       <c r="K92" t="n">
-        <v>547</v>
+        <v>432</v>
       </c>
     </row>
     <row r="93" ht="14.25" customHeight="1" s="250">
@@ -6327,7 +6327,7 @@
         <v>150000</v>
       </c>
       <c r="K97" t="n">
-        <v>8307</v>
+        <v>6559</v>
       </c>
     </row>
     <row r="98" ht="14.25" customHeight="1" s="250">
@@ -6477,7 +6477,7 @@
         <v>80000</v>
       </c>
       <c r="K101" t="n">
-        <v>4618</v>
+        <v>3646</v>
       </c>
     </row>
     <row r="102" ht="14.25" customHeight="1" s="250">
@@ -6516,7 +6516,7 @@
         <v>40000</v>
       </c>
       <c r="K102" t="n">
-        <v>2313</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="103" ht="14.25" customHeight="1" s="250">
@@ -6555,7 +6555,7 @@
         <v>26000</v>
       </c>
       <c r="K103" t="n">
-        <v>1192</v>
+        <v>941</v>
       </c>
     </row>
     <row r="104" ht="14.25" customHeight="1" s="250">
@@ -6633,7 +6633,7 @@
         <v>180000</v>
       </c>
       <c r="K105" t="n">
-        <v>9754</v>
+        <v>7701</v>
       </c>
     </row>
     <row r="106" ht="14.25" customHeight="1" s="250">
@@ -6783,7 +6783,7 @@
         <v>80000</v>
       </c>
       <c r="K109" t="n">
-        <v>4587</v>
+        <v>3621</v>
       </c>
     </row>
     <row r="110" ht="14.25" customHeight="1" s="250">
@@ -6822,7 +6822,7 @@
         <v>45000</v>
       </c>
       <c r="K110" t="n">
-        <v>2428</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="111" ht="14.25" customHeight="1" s="250">
@@ -6861,7 +6861,7 @@
         <v>25000</v>
       </c>
       <c r="K111" t="n">
-        <v>1219</v>
+        <v>963</v>
       </c>
     </row>
     <row r="112" ht="14.25" customHeight="1" s="250">
@@ -6939,7 +6939,7 @@
         <v>180000</v>
       </c>
       <c r="K113" t="n">
-        <v>9270</v>
+        <v>7318</v>
       </c>
     </row>
     <row r="114" ht="14.25" customHeight="1" s="250">
@@ -6978,7 +6978,7 @@
         <v>65000</v>
       </c>
       <c r="K114" t="n">
-        <v>3223</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="115" ht="14.25" customHeight="1" s="250">
@@ -7017,7 +7017,7 @@
         <v>20000</v>
       </c>
       <c r="K115" t="n">
-        <v>1153</v>
+        <v>910</v>
       </c>
     </row>
     <row r="116" ht="14.25" customHeight="1" s="250">
@@ -7056,7 +7056,7 @@
         <v>25000</v>
       </c>
       <c r="K116" t="n">
-        <v>1359</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="117" ht="14.25" customHeight="1" s="250">
@@ -7251,7 +7251,7 @@
         <v>150000</v>
       </c>
       <c r="K121" t="n">
-        <v>7524</v>
+        <v>5940</v>
       </c>
     </row>
     <row r="122" ht="14.25" customHeight="1" s="250">
@@ -7290,7 +7290,7 @@
         <v>68000</v>
       </c>
       <c r="K122" t="n">
-        <v>3775</v>
+        <v>2981</v>
       </c>
     </row>
     <row r="123" ht="14.25" customHeight="1" s="250">
@@ -7329,7 +7329,7 @@
         <v>15000</v>
       </c>
       <c r="K123" t="n">
-        <v>920</v>
+        <v>726</v>
       </c>
     </row>
     <row r="124" ht="14.25" customHeight="1" s="250">
@@ -7368,7 +7368,7 @@
         <v>10000</v>
       </c>
       <c r="K124" t="n">
-        <v>596</v>
+        <v>470</v>
       </c>
     </row>
     <row r="125" ht="14.25" customHeight="1" s="250">
@@ -7407,7 +7407,7 @@
         <v>75000</v>
       </c>
       <c r="K125" t="n">
-        <v>4149</v>
+        <v>3276</v>
       </c>
     </row>
     <row r="126" ht="14.25" customHeight="1" s="250">
@@ -7446,7 +7446,7 @@
         <v>32000</v>
       </c>
       <c r="K126" t="n">
-        <v>1399</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="127" ht="14.25" customHeight="1" s="250">
@@ -7485,7 +7485,7 @@
         <v>10000</v>
       </c>
       <c r="K127" t="n">
-        <v>528</v>
+        <v>417</v>
       </c>
     </row>
     <row r="128" ht="14.25" customHeight="1" s="250">
@@ -7563,7 +7563,7 @@
         <v>280000</v>
       </c>
       <c r="K129" t="n">
-        <v>15035</v>
+        <v>11870</v>
       </c>
     </row>
     <row r="130" ht="14.25" customHeight="1" s="250">
@@ -7604,7 +7604,7 @@
         <v>20000</v>
       </c>
       <c r="K130" t="n">
-        <v>921</v>
+        <v>727</v>
       </c>
     </row>
     <row r="131" ht="14.25" customHeight="1" s="250">
@@ -7645,7 +7645,7 @@
         <v>10000</v>
       </c>
       <c r="K131" t="n">
-        <v>597</v>
+        <v>471</v>
       </c>
     </row>
     <row r="132" ht="14.25" customHeight="1" s="250">
@@ -7686,7 +7686,7 @@
         <v>10000</v>
       </c>
       <c r="K132" t="n">
-        <v>595</v>
+        <v>469</v>
       </c>
     </row>
     <row r="133" ht="14.25" customHeight="1" s="250">
@@ -7727,7 +7727,7 @@
         <v>25000</v>
       </c>
       <c r="K133" t="n">
-        <v>1289</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="134" ht="14.25" customHeight="1" s="250">
@@ -7768,7 +7768,7 @@
         <v>15000</v>
       </c>
       <c r="K134" t="n">
-        <v>713</v>
+        <v>563</v>
       </c>
     </row>
     <row r="135" ht="14.25" customHeight="1" s="250">
@@ -7809,7 +7809,7 @@
         <v>10000</v>
       </c>
       <c r="K135" t="n">
-        <v>531</v>
+        <v>419</v>
       </c>
     </row>
     <row r="136" ht="14.25" customHeight="1" s="250">
@@ -7889,7 +7889,7 @@
         <v>140000</v>
       </c>
       <c r="K137" t="n">
-        <v>7138</v>
+        <v>5635</v>
       </c>
     </row>
     <row r="138" ht="14.25" customHeight="1" s="250">
@@ -7928,7 +7928,7 @@
         <v>20000</v>
       </c>
       <c r="K138" t="n">
-        <v>923</v>
+        <v>728</v>
       </c>
     </row>
     <row r="139" ht="14.25" customHeight="1" s="250">
@@ -7967,7 +7967,7 @@
         <v>10000</v>
       </c>
       <c r="K139" t="n">
-        <v>583</v>
+        <v>461</v>
       </c>
     </row>
     <row r="140" ht="14.25" customHeight="1" s="250">
@@ -8006,7 +8006,7 @@
         <v>10000</v>
       </c>
       <c r="K140" t="n">
-        <v>651</v>
+        <v>514</v>
       </c>
     </row>
     <row r="141" ht="14.25" customHeight="1" s="250">
@@ -8045,7 +8045,7 @@
         <v>30000</v>
       </c>
       <c r="K141" t="n">
-        <v>1550</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="142" ht="14.25" customHeight="1" s="250">
@@ -8084,7 +8084,7 @@
         <v>15000</v>
       </c>
       <c r="K142" t="n">
-        <v>819</v>
+        <v>647</v>
       </c>
     </row>
     <row r="143" ht="14.25" customHeight="1" s="250">
@@ -8123,7 +8123,7 @@
         <v>15000</v>
       </c>
       <c r="K143" t="n">
-        <v>883</v>
+        <v>697</v>
       </c>
     </row>
     <row r="144" ht="14.25" customHeight="1" s="250">
@@ -8201,7 +8201,7 @@
         <v>150000</v>
       </c>
       <c r="K145" t="n">
-        <v>8204</v>
+        <v>6477</v>
       </c>
     </row>
     <row r="146" ht="14.25" customHeight="1" s="250">
@@ -8240,7 +8240,7 @@
         <v>35000</v>
       </c>
       <c r="K146" t="n">
-        <v>1913</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="147" ht="14.25" customHeight="1" s="250">
@@ -8279,7 +8279,7 @@
         <v>10000</v>
       </c>
       <c r="K147" t="n">
-        <v>609</v>
+        <v>481</v>
       </c>
     </row>
     <row r="148" ht="14.25" customHeight="1" s="250">
@@ -8318,7 +8318,7 @@
         <v>12500</v>
       </c>
       <c r="K148" t="n">
-        <v>764</v>
+        <v>603</v>
       </c>
     </row>
     <row r="149" ht="14.25" customHeight="1" s="250">
@@ -8357,7 +8357,7 @@
         <v>40000</v>
       </c>
       <c r="K149" t="n">
-        <v>2134</v>
+        <v>1685</v>
       </c>
     </row>
     <row r="150" ht="14.25" customHeight="1" s="250">
@@ -8396,7 +8396,7 @@
         <v>20000</v>
       </c>
       <c r="K150" t="n">
-        <v>1023</v>
+        <v>808</v>
       </c>
     </row>
     <row r="151" ht="14.25" customHeight="1" s="250">
@@ -8435,7 +8435,7 @@
         <v>15000</v>
       </c>
       <c r="K151" t="n">
-        <v>780</v>
+        <v>616</v>
       </c>
     </row>
     <row r="152" ht="14.25" customHeight="1" s="250">
@@ -8513,7 +8513,7 @@
         <v>150000</v>
       </c>
       <c r="K153" t="n">
-        <v>7781</v>
+        <v>6143</v>
       </c>
     </row>
     <row r="154" ht="14.25" customHeight="1" s="250">
@@ -8552,7 +8552,7 @@
         <v>30000</v>
       </c>
       <c r="K154" t="n">
-        <v>1600</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="155" ht="14.25" customHeight="1" s="250">
@@ -8591,7 +8591,7 @@
         <v>10000</v>
       </c>
       <c r="K155" t="n">
-        <v>535</v>
+        <v>422</v>
       </c>
     </row>
     <row r="156" ht="14.25" customHeight="1" s="250">
@@ -8630,7 +8630,7 @@
         <v>10000</v>
       </c>
       <c r="K156" t="n">
-        <v>519</v>
+        <v>410</v>
       </c>
     </row>
     <row r="157" ht="14.25" customHeight="1" s="250">
@@ -8825,7 +8825,7 @@
         <v>120000</v>
       </c>
       <c r="K161" t="n">
-        <v>5546</v>
+        <v>4379</v>
       </c>
     </row>
     <row r="162" ht="14.25" customHeight="1" s="250">
@@ -8975,7 +8975,7 @@
         <v>65000</v>
       </c>
       <c r="K165" t="n">
-        <v>4333</v>
+        <v>3421</v>
       </c>
     </row>
     <row r="166" ht="14.25" customHeight="1" s="250">
@@ -9014,7 +9014,7 @@
         <v>38000</v>
       </c>
       <c r="K166" t="n">
-        <v>2533</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="167" ht="14.25" customHeight="1" s="250">
@@ -9053,7 +9053,7 @@
         <v>28000</v>
       </c>
       <c r="K167" t="n">
-        <v>1867</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="168" ht="14.25" customHeight="1" s="250">
@@ -9131,7 +9131,7 @@
         <v>167000</v>
       </c>
       <c r="K169" t="n">
-        <v>11133</v>
+        <v>8789</v>
       </c>
     </row>
     <row r="170" ht="14.25" customHeight="1" s="250">
@@ -9170,7 +9170,7 @@
         <v>745000</v>
       </c>
       <c r="K170" t="n">
-        <v>48330</v>
+        <v>38155</v>
       </c>
     </row>
     <row r="171" ht="14.25" customHeight="1" s="250">
@@ -9209,7 +9209,7 @@
         <v>180000</v>
       </c>
       <c r="K171" t="n">
-        <v>9814</v>
+        <v>7748</v>
       </c>
     </row>
     <row r="172" ht="14.25" customHeight="1" s="250">
@@ -9248,7 +9248,7 @@
         <v>135000</v>
       </c>
       <c r="K172" t="n">
-        <v>8826</v>
+        <v>6968</v>
       </c>
     </row>
     <row r="173" ht="14.25" customHeight="1" s="250">
@@ -9287,7 +9287,7 @@
         <v>1850000</v>
       </c>
       <c r="K173" t="n">
-        <v>121015</v>
+        <v>95538</v>
       </c>
     </row>
     <row r="174" ht="14.25" customHeight="1" s="250">
@@ -9326,7 +9326,7 @@
         <v>95000</v>
       </c>
       <c r="K174" t="n">
-        <v>5282</v>
+        <v>4170</v>
       </c>
     </row>
     <row r="175" ht="14.25" customHeight="1" s="250">
@@ -9365,7 +9365,7 @@
         <v>95000</v>
       </c>
       <c r="K175" t="n">
-        <v>5960</v>
+        <v>4705</v>
       </c>
     </row>
     <row r="176" ht="14.25" customHeight="1" s="250">
@@ -9443,7 +9443,7 @@
         <v>4260000</v>
       </c>
       <c r="K177" t="n">
-        <v>267307</v>
+        <v>211032</v>
       </c>
     </row>
     <row r="178" ht="14.25" customHeight="1" s="250">
@@ -9482,7 +9482,7 @@
         <v>320000</v>
       </c>
       <c r="K178" t="n">
-        <v>18537</v>
+        <v>14635</v>
       </c>
     </row>
     <row r="179" ht="14.25" customHeight="1" s="250">
@@ -9521,7 +9521,7 @@
         <v>80000</v>
       </c>
       <c r="K179" t="n">
-        <v>4604</v>
+        <v>3635</v>
       </c>
     </row>
     <row r="180" ht="14.25" customHeight="1" s="250">
@@ -9560,7 +9560,7 @@
         <v>116000</v>
       </c>
       <c r="K180" t="n">
-        <v>7156</v>
+        <v>5650</v>
       </c>
     </row>
     <row r="181" ht="14.25" customHeight="1" s="250">
@@ -9599,7 +9599,7 @@
         <v>318000</v>
       </c>
       <c r="K181" t="n">
-        <v>17704</v>
+        <v>13977</v>
       </c>
     </row>
     <row r="182" ht="14.25" customHeight="1" s="250">
@@ -9638,7 +9638,7 @@
         <v>182000</v>
       </c>
       <c r="K182" t="n">
-        <v>10070</v>
+        <v>7950</v>
       </c>
     </row>
     <row r="183" ht="14.25" customHeight="1" s="250">
@@ -9677,7 +9677,7 @@
         <v>109000</v>
       </c>
       <c r="K183" t="n">
-        <v>6073</v>
+        <v>4795</v>
       </c>
     </row>
     <row r="184" ht="14.25" customHeight="1" s="250">
@@ -9755,7 +9755,7 @@
         <v>1513000</v>
       </c>
       <c r="K185" t="n">
-        <v>84981</v>
+        <v>67090</v>
       </c>
     </row>
     <row r="186" ht="14.25" customHeight="1" s="250">
@@ -9833,7 +9833,7 @@
         <v>7440000</v>
       </c>
       <c r="K187" t="n">
-        <v>441982</v>
+        <v>348933</v>
       </c>
     </row>
     <row r="188" ht="14.25" customHeight="1" s="250">
@@ -9872,7 +9872,7 @@
         <v>3600000</v>
       </c>
       <c r="K188" t="n">
-        <v>218620</v>
+        <v>172594</v>
       </c>
     </row>
     <row r="189" ht="14.25" customHeight="1" s="250">
@@ -9911,7 +9911,7 @@
         <v>3800000</v>
       </c>
       <c r="K189" t="n">
-        <v>229387</v>
+        <v>181095</v>
       </c>
     </row>
     <row r="190" ht="14.25" customHeight="1" s="250">
@@ -10221,10 +10221,10 @@
         <v>0.159622112638379</v>
       </c>
       <c r="H2" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="I2" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -10252,10 +10252,10 @@
         <v>0.13006246214979</v>
       </c>
       <c r="H3" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I3" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="13.5" customHeight="1" s="250">
@@ -10283,10 +10283,10 @@
         <v>0.12785218855059</v>
       </c>
       <c r="H4" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="I4" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="250">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="G5" s="258" t="n"/>
       <c r="I5" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="250">
@@ -10338,10 +10338,10 @@
         <v>0.119182965859955</v>
       </c>
       <c r="H6" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="I6" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="250" thickBot="1">
@@ -10369,10 +10369,10 @@
         <v>0.106909295617267</v>
       </c>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="I7" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" ht="30" customFormat="1" customHeight="1" s="158">
@@ -10400,10 +10400,10 @@
         <v>0.127185196510197</v>
       </c>
       <c r="H8" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="I8" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="250">
@@ -10431,10 +10431,10 @@
         <v>0.130798384540069</v>
       </c>
       <c r="H9" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I9" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="250">
@@ -10462,10 +10462,10 @@
         <v>0.197218920214015</v>
       </c>
       <c r="H10" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="250">
@@ -10493,10 +10493,10 @@
         <v>0.156143076621019</v>
       </c>
       <c r="H11" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="I11" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="250">
@@ -10524,10 +10524,10 @@
         <v>0.125550416455854</v>
       </c>
       <c r="H12" t="n">
-        <v>305</v>
+        <v>241</v>
       </c>
       <c r="I12" t="n">
-        <v>277</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="250">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="G13" s="258" t="n"/>
       <c r="I13" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="250">
@@ -10579,10 +10579,10 @@
         <v>0.0806766817717267</v>
       </c>
       <c r="H14" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I14" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="250">
@@ -10610,10 +10610,10 @@
         <v>0.0777021675916213</v>
       </c>
       <c r="H15" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="I15" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="250">
@@ -10637,7 +10637,7 @@
       </c>
       <c r="G16" s="260" t="n"/>
       <c r="I16" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="250">
@@ -10665,10 +10665,10 @@
         <v>0.095303991140541</v>
       </c>
       <c r="H17" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="I17" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="250">
@@ -10696,10 +10696,10 @@
         <v>0.0776551038922926</v>
       </c>
       <c r="H18" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I18" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="250">
@@ -10727,10 +10727,10 @@
         <v>0.162114464314885</v>
       </c>
       <c r="H19" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I19" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="250">
@@ -10754,7 +10754,7 @@
       </c>
       <c r="G20" s="208" t="n"/>
       <c r="I20" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="250">
@@ -10782,10 +10782,10 @@
         <v>0.08919891687813671</v>
       </c>
       <c r="H21" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I21" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="250">
@@ -10813,10 +10813,10 @@
         <v>0.08301513631583469</v>
       </c>
       <c r="H22" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="I22" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="250">
@@ -10844,10 +10844,10 @@
         <v>0.06665486782805979</v>
       </c>
       <c r="H23" t="n">
-        <v>381</v>
+        <v>301</v>
       </c>
       <c r="I23" t="n">
-        <v>362</v>
+        <v>285</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="250">
@@ -10875,10 +10875,10 @@
         <v>0.07487484353666519</v>
       </c>
       <c r="H24" t="n">
-        <v>734</v>
+        <v>580</v>
       </c>
       <c r="I24" t="n">
-        <v>677</v>
+        <v>534</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="250">

</xml_diff>